<commit_message>
chore(data): daily snapshot 2026-06-22
</commit_message>
<xml_diff>
--- a/projects/mobile-price-tracker/data/mobile_plans.xlsx
+++ b/projects/mobile-price-tracker/data/mobile_plans.xlsx
@@ -1554,7 +1554,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -1980,7 +1980,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -2774,7 +2774,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -3332,7 +3332,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -3534,7 +3534,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3884,7 +3884,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -3950,7 +3950,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -4144,7 +4144,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -4424,7 +4424,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -4498,7 +4498,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -4646,7 +4646,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -4716,7 +4716,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -4782,7 +4782,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -4848,7 +4848,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -5120,7 +5120,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -5196,7 +5196,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -5266,7 +5266,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -5336,7 +5336,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -5406,7 +5406,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -5476,7 +5476,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -5616,7 +5616,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -5756,7 +5756,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -5826,7 +5826,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -5896,7 +5896,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -5966,7 +5966,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -6094,7 +6094,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -6156,7 +6156,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -6218,7 +6218,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -6340,7 +6340,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -6526,7 +6526,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -6588,7 +6588,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -6712,7 +6712,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -6774,7 +6774,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -6836,7 +6836,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -6898,7 +6898,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -6960,7 +6960,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -7030,7 +7030,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -7240,7 +7240,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -7310,7 +7310,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -7380,7 +7380,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -7450,7 +7450,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -7516,7 +7516,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -7582,7 +7582,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -7648,7 +7648,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -7710,7 +7710,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -7772,7 +7772,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -7842,7 +7842,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -7916,7 +7916,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -7990,7 +7990,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -8138,7 +8138,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -8212,7 +8212,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -8282,7 +8282,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -8480,7 +8480,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -8666,7 +8666,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): daily snapshot 2026-06-24
</commit_message>
<xml_diff>
--- a/projects/mobile-price-tracker/data/mobile_plans.xlsx
+++ b/projects/mobile-price-tracker/data/mobile_plans.xlsx
@@ -18,7 +18,7 @@
     <sheet name="TIM" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'history'!$A$1:$T$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'history'!$A$1:$T$150</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'latest'!$A$1:$T$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -296,12 +296,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$38</f>
+              <f>'comparison'!$A$37:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$B$37:$B$38</f>
+              <f>'comparison'!$B$37:$B$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -333,12 +333,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$38</f>
+              <f>'comparison'!$A$37:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$C$37:$C$38</f>
+              <f>'comparison'!$C$37:$C$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -370,12 +370,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$38</f>
+              <f>'comparison'!$A$37:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$D$37:$D$38</f>
+              <f>'comparison'!$D$37:$D$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -493,12 +493,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$38</f>
+              <f>'comparison'!$A$37:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$E$37:$E$38</f>
+              <f>'comparison'!$E$37:$E$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -530,12 +530,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$38</f>
+              <f>'comparison'!$A$37:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$F$37:$F$38</f>
+              <f>'comparison'!$F$37:$F$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -567,12 +567,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$38</f>
+              <f>'comparison'!$A$37:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$G$37:$G$38</f>
+              <f>'comparison'!$G$37:$G$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -690,12 +690,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$38</f>
+              <f>'comparison'!$A$37:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$H$37:$H$38</f>
+              <f>'comparison'!$H$37:$H$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -727,12 +727,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$38</f>
+              <f>'comparison'!$A$37:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$I$37:$I$38</f>
+              <f>'comparison'!$I$37:$I$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -764,12 +764,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$38</f>
+              <f>'comparison'!$A$37:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$J$37:$J$38</f>
+              <f>'comparison'!$J$37:$J$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -887,12 +887,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$38</f>
+              <f>'comparison'!$A$37:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$K$37:$K$38</f>
+              <f>'comparison'!$K$37:$K$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -924,12 +924,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$38</f>
+              <f>'comparison'!$A$37:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$L$37:$L$38</f>
+              <f>'comparison'!$L$37:$L$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -961,12 +961,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$38</f>
+              <f>'comparison'!$A$37:$A$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$M$37:$M$38</f>
+              <f>'comparison'!$M$37:$M$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1419,7 +1419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T101"/>
+  <dimension ref="A1:T150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -8286,8 +8286,3322 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>Controle 25GB</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>claro:plano-controle-25gb</t>
+        </is>
+      </c>
+      <c r="H102" s="3" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="I102" s="3" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>De R$ 59,90 Por:</t>
+        </is>
+      </c>
+      <c r="K102" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="L102" s="2" t="inlineStr"/>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N102" s="2" t="inlineStr"/>
+      <c r="O102" s="2" t="inlineStr"/>
+      <c r="P102" s="2" t="inlineStr"/>
+      <c r="Q102" s="2" t="inlineStr"/>
+      <c r="R102" s="2" t="inlineStr">
+        <is>
+          <t>Para uso livre; Para redes sociais e vídeos; Bônus exclusivo; Aproveite na sua franquia; WhatsApp e ligações ilimitadas</t>
+        </is>
+      </c>
+      <c r="S102" s="2" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/controle</t>
+        </is>
+      </c>
+      <c r="T102" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/claro_control_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>Controle 30GB</t>
+        </is>
+      </c>
+      <c r="G103" s="5" t="inlineStr">
+        <is>
+          <t>claro:plano-controle-30gb</t>
+        </is>
+      </c>
+      <c r="H103" s="6" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="I103" s="6" t="inlineStr"/>
+      <c r="J103" s="5" t="inlineStr"/>
+      <c r="K103" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="L103" s="5" t="inlineStr"/>
+      <c r="M103" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N103" s="5" t="inlineStr"/>
+      <c r="O103" s="5" t="inlineStr"/>
+      <c r="P103" s="5" t="inlineStr"/>
+      <c r="Q103" s="5" t="inlineStr"/>
+      <c r="R103" s="5" t="inlineStr">
+        <is>
+          <t>Para uso livre; Bônus do Hexa para uso livre; Bônus para redes sociais e apps; Redes sociais e apps; WhatsApp ilimitado</t>
+        </is>
+      </c>
+      <c r="S103" s="5" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/controle</t>
+        </is>
+      </c>
+      <c r="T103" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/claro_control_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Controle 30GB</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>claro:plano-controle-30gb-gaming</t>
+        </is>
+      </c>
+      <c r="H104" s="3" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="I104" s="3" t="inlineStr"/>
+      <c r="J104" s="2" t="inlineStr"/>
+      <c r="K104" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="L104" s="2" t="inlineStr"/>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N104" s="2" t="inlineStr"/>
+      <c r="O104" s="2" t="inlineStr"/>
+      <c r="P104" s="2" t="inlineStr"/>
+      <c r="Q104" s="2" t="inlineStr"/>
+      <c r="R104" s="2" t="inlineStr">
+        <is>
+          <t>Para uso livre; Bônus para redes sociais e apps; Bônus uso livre; Redes sociais e apps; WhatsApp ilimitado</t>
+        </is>
+      </c>
+      <c r="S104" s="2" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/controle</t>
+        </is>
+      </c>
+      <c r="T104" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/claro_control_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>flex</t>
+        </is>
+      </c>
+      <c r="E105" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F105" s="5" t="inlineStr">
+        <is>
+          <t>Flex 15GB</t>
+        </is>
+      </c>
+      <c r="G105" s="5" t="inlineStr">
+        <is>
+          <t>claro:plano-flex-15gb</t>
+        </is>
+      </c>
+      <c r="H105" s="6" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="I105" s="6" t="inlineStr"/>
+      <c r="J105" s="5" t="inlineStr"/>
+      <c r="K105" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="L105" s="5" t="inlineStr"/>
+      <c r="M105" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N105" s="5" t="inlineStr"/>
+      <c r="O105" s="5" t="inlineStr"/>
+      <c r="P105" s="5" t="inlineStr"/>
+      <c r="Q105" s="5" t="inlineStr"/>
+      <c r="R105" s="5" t="inlineStr">
+        <is>
+          <t>Para uso livre; Bônus do Hexa para uso livre; Para redes sociais e apps; Bônus extra nos apps; WhatsApp ilimitado</t>
+        </is>
+      </c>
+      <c r="S105" s="5" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/flex</t>
+        </is>
+      </c>
+      <c r="T105" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/claro_flex_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>flex</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>Flex 20GB</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>claro:plano-flex-20gb</t>
+        </is>
+      </c>
+      <c r="H106" s="3" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="I106" s="3" t="inlineStr"/>
+      <c r="J106" s="2" t="inlineStr"/>
+      <c r="K106" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="L106" s="2" t="inlineStr"/>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N106" s="2" t="inlineStr"/>
+      <c r="O106" s="2" t="inlineStr"/>
+      <c r="P106" s="2" t="inlineStr"/>
+      <c r="Q106" s="2" t="inlineStr"/>
+      <c r="R106" s="2" t="inlineStr">
+        <is>
+          <t>Para uso livre; Bônus do Hexa para uso livre; Para redes sociais e apps; Bônus extra nos apps; WhatsApp ilimitado</t>
+        </is>
+      </c>
+      <c r="S106" s="2" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/flex</t>
+        </is>
+      </c>
+      <c r="T106" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/claro_flex_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>flex</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F107" s="5" t="inlineStr">
+        <is>
+          <t>Flex 30GB</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="inlineStr">
+        <is>
+          <t>claro:plano-flex-30gb</t>
+        </is>
+      </c>
+      <c r="H107" s="6" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="I107" s="6" t="inlineStr"/>
+      <c r="J107" s="5" t="inlineStr"/>
+      <c r="K107" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="L107" s="5" t="inlineStr"/>
+      <c r="M107" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N107" s="5" t="inlineStr"/>
+      <c r="O107" s="5" t="inlineStr"/>
+      <c r="P107" s="5" t="inlineStr"/>
+      <c r="Q107" s="5" t="inlineStr"/>
+      <c r="R107" s="5" t="inlineStr">
+        <is>
+          <t>Para uso livre; Bônus do Hexa para uso livre; Para redes sociais e apps; Bônus extra nos apps; WhatsApp ilimitado; Assinatura Claro musica inclusa</t>
+        </is>
+      </c>
+      <c r="S107" s="5" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/flex</t>
+        </is>
+      </c>
+      <c r="T107" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/claro_flex_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>flex</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Flex 40GB</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>claro:plano-flex-40gb</t>
+        </is>
+      </c>
+      <c r="H108" s="3" t="n">
+        <v>119.9</v>
+      </c>
+      <c r="I108" s="3" t="inlineStr"/>
+      <c r="J108" s="2" t="inlineStr"/>
+      <c r="K108" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="L108" s="2" t="inlineStr"/>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N108" s="2" t="inlineStr"/>
+      <c r="O108" s="2" t="inlineStr"/>
+      <c r="P108" s="2" t="inlineStr"/>
+      <c r="Q108" s="2" t="inlineStr"/>
+      <c r="R108" s="2" t="inlineStr">
+        <is>
+          <t>Para uso livre; Para redes sociais e apps; Bônus uso livre; Bônus extra nos apps; WhatsApp ilimitado; Assinatura Claro musica inclusa</t>
+        </is>
+      </c>
+      <c r="S108" s="2" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/flex</t>
+        </is>
+      </c>
+      <c r="T108" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/claro_flex_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F109" s="5" t="inlineStr">
+        <is>
+          <t>Pós 100GB</t>
+        </is>
+      </c>
+      <c r="G109" s="5" t="inlineStr">
+        <is>
+          <t>claro:plano-pos-100gb</t>
+        </is>
+      </c>
+      <c r="H109" s="6" t="n">
+        <v>179.9</v>
+      </c>
+      <c r="I109" s="6" t="inlineStr"/>
+      <c r="J109" s="5" t="inlineStr"/>
+      <c r="K109" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L109" s="5" t="inlineStr"/>
+      <c r="M109" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N109" s="5" t="inlineStr"/>
+      <c r="O109" s="5" t="inlineStr"/>
+      <c r="P109" s="5" t="inlineStr"/>
+      <c r="Q109" s="5" t="inlineStr"/>
+      <c r="R109" s="5" t="inlineStr">
+        <is>
+          <t>Armazenamento na nuvem:; Google One ou iCloud+; WhatsApp ilimitado; Roaming: Passaporte Américas; Claro Sync: Smartwatch conectado</t>
+        </is>
+      </c>
+      <c r="S109" s="5" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/pos</t>
+        </is>
+      </c>
+      <c r="T109" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/claro_postpaid_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>Pós 150GB</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>claro:plano-pos-150gb</t>
+        </is>
+      </c>
+      <c r="H110" s="3" t="n">
+        <v>239.9</v>
+      </c>
+      <c r="I110" s="3" t="inlineStr"/>
+      <c r="J110" s="2" t="inlineStr"/>
+      <c r="K110" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="L110" s="2" t="inlineStr"/>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N110" s="2" t="inlineStr"/>
+      <c r="O110" s="2" t="inlineStr"/>
+      <c r="P110" s="2" t="inlineStr"/>
+      <c r="Q110" s="2" t="inlineStr"/>
+      <c r="R110" s="2" t="inlineStr">
+        <is>
+          <t>Armazenamento na nuvem:; Google One ou iCloud+; WhatsApp ilimitado; Roaming: Passaporte Américas e Europa; Claro Sync: Smartwatch conectado</t>
+        </is>
+      </c>
+      <c r="S110" s="2" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/pos</t>
+        </is>
+      </c>
+      <c r="T110" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/claro_postpaid_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F111" s="5" t="inlineStr">
+        <is>
+          <t>Pós 200GB</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr">
+        <is>
+          <t>claro:plano-pos-200gb</t>
+        </is>
+      </c>
+      <c r="H111" s="6" t="n">
+        <v>339.9</v>
+      </c>
+      <c r="I111" s="6" t="inlineStr"/>
+      <c r="J111" s="5" t="inlineStr"/>
+      <c r="K111" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="L111" s="5" t="inlineStr"/>
+      <c r="M111" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N111" s="5" t="inlineStr"/>
+      <c r="O111" s="5" t="inlineStr"/>
+      <c r="P111" s="5" t="inlineStr"/>
+      <c r="Q111" s="5" t="inlineStr"/>
+      <c r="R111" s="5" t="inlineStr">
+        <is>
+          <t>Armazenamento na nuvem:; Google One ou iCloud+; WhatsApp ilimitado; Roaming: Passaporte Mundo; Claro Sync: Smartwatch conectado</t>
+        </is>
+      </c>
+      <c r="S111" s="5" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/pos</t>
+        </is>
+      </c>
+      <c r="T111" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/claro_postpaid_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Pós 50GB com GeForce NOW</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>claro:plano-pos-60gb-geforce</t>
+        </is>
+      </c>
+      <c r="H112" s="3" t="n">
+        <v>164.9</v>
+      </c>
+      <c r="I112" s="3" t="inlineStr"/>
+      <c r="J112" s="2" t="inlineStr"/>
+      <c r="K112" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="L112" s="2" t="inlineStr"/>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N112" s="2" t="inlineStr"/>
+      <c r="O112" s="2" t="inlineStr"/>
+      <c r="P112" s="2" t="inlineStr"/>
+      <c r="Q112" s="2" t="inlineStr"/>
+      <c r="R112" s="2" t="inlineStr">
+        <is>
+          <t>Armazenamento na nuvem:; Google One ou iCloud+; WhatsApp ilimitado; Roaming: Passaporte Américas; Claro Sync: Smartwatch conectado; Inclusa assinatura GeForce NOW</t>
+        </is>
+      </c>
+      <c r="S112" s="2" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/pos</t>
+        </is>
+      </c>
+      <c r="T112" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/claro_postpaid_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>Pós 60GB</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>claro:plano-pos-60gb</t>
+        </is>
+      </c>
+      <c r="H113" s="6" t="n">
+        <v>124.9</v>
+      </c>
+      <c r="I113" s="6" t="inlineStr"/>
+      <c r="J113" s="5" t="inlineStr"/>
+      <c r="K113" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="L113" s="5" t="inlineStr"/>
+      <c r="M113" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N113" s="5" t="inlineStr"/>
+      <c r="O113" s="5" t="inlineStr"/>
+      <c r="P113" s="5" t="inlineStr"/>
+      <c r="Q113" s="5" t="inlineStr"/>
+      <c r="R113" s="5" t="inlineStr">
+        <is>
+          <t>Armazenamento na nuvem:; Google One ou iCloud+; WhatsApp ilimitado; Roaming: Passaporte Américas; Claro Sync: Smartwatch conectado</t>
+        </is>
+      </c>
+      <c r="S113" s="5" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/pos</t>
+        </is>
+      </c>
+      <c r="T113" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/claro_postpaid_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>Prezão R$1 por dia</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>claro:prez-o-r-1-por-dia</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I114" s="3" t="inlineStr"/>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>prepaid Prezão — preço por dia; recargas a partir de R$15</t>
+        </is>
+      </c>
+      <c r="K114" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L114" s="2" t="inlineStr"/>
+      <c r="M114" s="2" t="inlineStr"/>
+      <c r="N114" s="2" t="inlineStr"/>
+      <c r="O114" s="2" t="inlineStr"/>
+      <c r="P114" s="2" t="inlineStr"/>
+      <c r="Q114" s="2" t="inlineStr"/>
+      <c r="R114" s="2" t="inlineStr"/>
+      <c r="S114" s="2" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/planos-pre/prezao</t>
+        </is>
+      </c>
+      <c r="T114" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/claro_prepaid_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>TIM Controle 41GB</t>
+        </is>
+      </c>
+      <c r="G115" s="5" t="inlineStr">
+        <is>
+          <t>tim:162901</t>
+        </is>
+      </c>
+      <c r="H115" s="6" t="n">
+        <v>58.99</v>
+      </c>
+      <c r="I115" s="6" t="inlineStr"/>
+      <c r="J115" s="5" t="inlineStr"/>
+      <c r="K115" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="L115" s="5" t="inlineStr"/>
+      <c r="M115" s="5" t="inlineStr"/>
+      <c r="N115" s="5" t="inlineStr"/>
+      <c r="O115" s="5" t="inlineStr"/>
+      <c r="P115" s="5" t="inlineStr"/>
+      <c r="Q115" s="5" t="inlineStr"/>
+      <c r="R115" s="5" t="inlineStr"/>
+      <c r="S115" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/controle</t>
+        </is>
+      </c>
+      <c r="T115" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>TIM Controle Light Express 31GB</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>tim:143536</t>
+        </is>
+      </c>
+      <c r="H116" s="3" t="n">
+        <v>60.99</v>
+      </c>
+      <c r="I116" s="3" t="inlineStr"/>
+      <c r="J116" s="2" t="inlineStr"/>
+      <c r="K116" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="L116" s="2" t="inlineStr"/>
+      <c r="M116" s="2" t="inlineStr"/>
+      <c r="N116" s="2" t="inlineStr"/>
+      <c r="O116" s="2" t="inlineStr"/>
+      <c r="P116" s="2" t="inlineStr"/>
+      <c r="Q116" s="2" t="inlineStr"/>
+      <c r="R116" s="2" t="inlineStr"/>
+      <c r="S116" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/controle</t>
+        </is>
+      </c>
+      <c r="T116" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F117" s="5" t="inlineStr">
+        <is>
+          <t>TIM Controle Plus 45GB</t>
+        </is>
+      </c>
+      <c r="G117" s="5" t="inlineStr">
+        <is>
+          <t>tim:155891</t>
+        </is>
+      </c>
+      <c r="H117" s="6" t="n">
+        <v>64.98999999999999</v>
+      </c>
+      <c r="I117" s="6" t="inlineStr"/>
+      <c r="J117" s="5" t="inlineStr"/>
+      <c r="K117" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="L117" s="5" t="inlineStr"/>
+      <c r="M117" s="5" t="inlineStr"/>
+      <c r="N117" s="5" t="inlineStr"/>
+      <c r="O117" s="5" t="inlineStr"/>
+      <c r="P117" s="5" t="inlineStr"/>
+      <c r="Q117" s="5" t="inlineStr"/>
+      <c r="R117" s="5" t="inlineStr"/>
+      <c r="S117" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/controle</t>
+        </is>
+      </c>
+      <c r="T117" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>TIM Controle Premium 53GB</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>tim:162896</t>
+        </is>
+      </c>
+      <c r="H118" s="3" t="n">
+        <v>84.98999999999999</v>
+      </c>
+      <c r="I118" s="3" t="inlineStr"/>
+      <c r="J118" s="2" t="inlineStr"/>
+      <c r="K118" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="L118" s="2" t="inlineStr"/>
+      <c r="M118" s="2" t="inlineStr"/>
+      <c r="N118" s="2" t="inlineStr"/>
+      <c r="O118" s="2" t="inlineStr"/>
+      <c r="P118" s="2" t="inlineStr"/>
+      <c r="Q118" s="2" t="inlineStr"/>
+      <c r="R118" s="2" t="inlineStr"/>
+      <c r="S118" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/controle</t>
+        </is>
+      </c>
+      <c r="T118" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F119" s="5" t="inlineStr">
+        <is>
+          <t>TIM Controle Pro Express</t>
+        </is>
+      </c>
+      <c r="G119" s="5" t="inlineStr">
+        <is>
+          <t>tim:143576</t>
+        </is>
+      </c>
+      <c r="H119" s="6" t="n">
+        <v>64.98999999999999</v>
+      </c>
+      <c r="I119" s="6" t="inlineStr"/>
+      <c r="J119" s="5" t="inlineStr"/>
+      <c r="K119" s="7" t="inlineStr"/>
+      <c r="L119" s="5" t="inlineStr"/>
+      <c r="M119" s="5" t="inlineStr"/>
+      <c r="N119" s="5" t="inlineStr"/>
+      <c r="O119" s="5" t="inlineStr"/>
+      <c r="P119" s="5" t="inlineStr"/>
+      <c r="Q119" s="5" t="inlineStr"/>
+      <c r="R119" s="5" t="inlineStr"/>
+      <c r="S119" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/controle</t>
+        </is>
+      </c>
+      <c r="T119" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>TIM Black 70GB</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>tim:54206</t>
+        </is>
+      </c>
+      <c r="H120" s="3" t="n">
+        <v>129.99</v>
+      </c>
+      <c r="I120" s="3" t="inlineStr"/>
+      <c r="J120" s="2" t="inlineStr"/>
+      <c r="K120" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="L120" s="2" t="inlineStr"/>
+      <c r="M120" s="2" t="inlineStr"/>
+      <c r="N120" s="2" t="inlineStr"/>
+      <c r="O120" s="2" t="inlineStr"/>
+      <c r="P120" s="2" t="inlineStr"/>
+      <c r="Q120" s="2" t="inlineStr"/>
+      <c r="R120" s="2" t="inlineStr"/>
+      <c r="S120" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pos-pago/tim-black</t>
+        </is>
+      </c>
+      <c r="T120" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D121" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F121" s="5" t="inlineStr">
+        <is>
+          <t>TIM Black A Express 67GB</t>
+        </is>
+      </c>
+      <c r="G121" s="5" t="inlineStr">
+        <is>
+          <t>tim:55121</t>
+        </is>
+      </c>
+      <c r="H121" s="6" t="n">
+        <v>119.99</v>
+      </c>
+      <c r="I121" s="6" t="inlineStr"/>
+      <c r="J121" s="5" t="inlineStr"/>
+      <c r="K121" s="7" t="n">
+        <v>67</v>
+      </c>
+      <c r="L121" s="5" t="inlineStr"/>
+      <c r="M121" s="5" t="inlineStr"/>
+      <c r="N121" s="5" t="inlineStr"/>
+      <c r="O121" s="5" t="inlineStr"/>
+      <c r="P121" s="5" t="inlineStr"/>
+      <c r="Q121" s="5" t="inlineStr"/>
+      <c r="R121" s="5" t="inlineStr"/>
+      <c r="S121" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pos-pago/tim-black</t>
+        </is>
+      </c>
+      <c r="T121" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>TIM Black B Express 82GB</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>tim:52146</t>
+        </is>
+      </c>
+      <c r="H122" s="3" t="n">
+        <v>144.99</v>
+      </c>
+      <c r="I122" s="3" t="inlineStr"/>
+      <c r="J122" s="2" t="inlineStr"/>
+      <c r="K122" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="L122" s="2" t="inlineStr"/>
+      <c r="M122" s="2" t="inlineStr"/>
+      <c r="N122" s="2" t="inlineStr"/>
+      <c r="O122" s="2" t="inlineStr"/>
+      <c r="P122" s="2" t="inlineStr"/>
+      <c r="Q122" s="2" t="inlineStr"/>
+      <c r="R122" s="2" t="inlineStr"/>
+      <c r="S122" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pos-pago/tim-black</t>
+        </is>
+      </c>
+      <c r="T122" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>TIM Black C Express 107GB</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>tim:52151</t>
+        </is>
+      </c>
+      <c r="H123" s="6" t="n">
+        <v>164.99</v>
+      </c>
+      <c r="I123" s="6" t="inlineStr"/>
+      <c r="J123" s="5" t="inlineStr"/>
+      <c r="K123" s="7" t="n">
+        <v>107</v>
+      </c>
+      <c r="L123" s="5" t="inlineStr"/>
+      <c r="M123" s="5" t="inlineStr"/>
+      <c r="N123" s="5" t="inlineStr"/>
+      <c r="O123" s="5" t="inlineStr"/>
+      <c r="P123" s="5" t="inlineStr"/>
+      <c r="Q123" s="5" t="inlineStr"/>
+      <c r="R123" s="5" t="inlineStr"/>
+      <c r="S123" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pos-pago/tim-black</t>
+        </is>
+      </c>
+      <c r="T123" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>TIM Black C Ultra 95GB</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>tim:100581</t>
+        </is>
+      </c>
+      <c r="H124" s="3" t="n">
+        <v>159.99</v>
+      </c>
+      <c r="I124" s="3" t="inlineStr"/>
+      <c r="J124" s="2" t="inlineStr"/>
+      <c r="K124" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="L124" s="2" t="inlineStr"/>
+      <c r="M124" s="2" t="inlineStr"/>
+      <c r="N124" s="2" t="inlineStr"/>
+      <c r="O124" s="2" t="inlineStr"/>
+      <c r="P124" s="2" t="inlineStr"/>
+      <c r="Q124" s="2" t="inlineStr"/>
+      <c r="R124" s="2" t="inlineStr"/>
+      <c r="S124" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pos-pago/tim-black</t>
+        </is>
+      </c>
+      <c r="T124" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>TIM Black Plus 80GB</t>
+        </is>
+      </c>
+      <c r="G125" s="5" t="inlineStr">
+        <is>
+          <t>tim:54256</t>
+        </is>
+      </c>
+      <c r="H125" s="6" t="n">
+        <v>149.99</v>
+      </c>
+      <c r="I125" s="6" t="inlineStr"/>
+      <c r="J125" s="5" t="inlineStr"/>
+      <c r="K125" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="L125" s="5" t="inlineStr"/>
+      <c r="M125" s="5" t="inlineStr"/>
+      <c r="N125" s="5" t="inlineStr"/>
+      <c r="O125" s="5" t="inlineStr"/>
+      <c r="P125" s="5" t="inlineStr"/>
+      <c r="Q125" s="5" t="inlineStr"/>
+      <c r="R125" s="5" t="inlineStr"/>
+      <c r="S125" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pos-pago/tim-black</t>
+        </is>
+      </c>
+      <c r="T125" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>TIM Black Premium 110GB</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>tim:54261</t>
+        </is>
+      </c>
+      <c r="H126" s="3" t="n">
+        <v>159.99</v>
+      </c>
+      <c r="I126" s="3" t="inlineStr"/>
+      <c r="J126" s="2" t="inlineStr"/>
+      <c r="K126" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="L126" s="2" t="inlineStr"/>
+      <c r="M126" s="2" t="inlineStr"/>
+      <c r="N126" s="2" t="inlineStr"/>
+      <c r="O126" s="2" t="inlineStr"/>
+      <c r="P126" s="2" t="inlineStr"/>
+      <c r="Q126" s="2" t="inlineStr"/>
+      <c r="R126" s="2" t="inlineStr"/>
+      <c r="S126" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pos-pago/tim-black</t>
+        </is>
+      </c>
+      <c r="T126" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D127" s="5" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E127" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F127" s="5" t="inlineStr">
+        <is>
+          <t>TIM Pré XIP Plus 16GB</t>
+        </is>
+      </c>
+      <c r="G127" s="5" t="inlineStr">
+        <is>
+          <t>tim:106306</t>
+        </is>
+      </c>
+      <c r="H127" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I127" s="6" t="inlineStr"/>
+      <c r="J127" s="5" t="inlineStr"/>
+      <c r="K127" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="L127" s="5" t="inlineStr"/>
+      <c r="M127" s="5" t="inlineStr"/>
+      <c r="N127" s="5" t="inlineStr"/>
+      <c r="O127" s="5" t="inlineStr"/>
+      <c r="P127" s="5" t="inlineStr"/>
+      <c r="Q127" s="5" t="inlineStr"/>
+      <c r="R127" s="5" t="inlineStr"/>
+      <c r="S127" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pre-pago</t>
+        </is>
+      </c>
+      <c r="T127" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_prepaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>TIM Pré XIP Plus 6GB</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>tim:59906</t>
+        </is>
+      </c>
+      <c r="H128" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I128" s="3" t="inlineStr"/>
+      <c r="J128" s="2" t="inlineStr"/>
+      <c r="K128" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L128" s="2" t="inlineStr"/>
+      <c r="M128" s="2" t="inlineStr"/>
+      <c r="N128" s="2" t="inlineStr"/>
+      <c r="O128" s="2" t="inlineStr"/>
+      <c r="P128" s="2" t="inlineStr"/>
+      <c r="Q128" s="2" t="inlineStr"/>
+      <c r="R128" s="2" t="inlineStr"/>
+      <c r="S128" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pre-pago</t>
+        </is>
+      </c>
+      <c r="T128" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_prepaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D129" s="5" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E129" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F129" s="5" t="inlineStr">
+        <is>
+          <t>TIM Pré XIP Plus 8GB</t>
+        </is>
+      </c>
+      <c r="G129" s="5" t="inlineStr">
+        <is>
+          <t>tim:59901</t>
+        </is>
+      </c>
+      <c r="H129" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="I129" s="6" t="inlineStr"/>
+      <c r="J129" s="5" t="inlineStr"/>
+      <c r="K129" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L129" s="5" t="inlineStr"/>
+      <c r="M129" s="5" t="inlineStr"/>
+      <c r="N129" s="5" t="inlineStr"/>
+      <c r="O129" s="5" t="inlineStr"/>
+      <c r="P129" s="5" t="inlineStr"/>
+      <c r="Q129" s="5" t="inlineStr"/>
+      <c r="R129" s="5" t="inlineStr"/>
+      <c r="S129" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pre-pago</t>
+        </is>
+      </c>
+      <c r="T129" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_prepaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029270-46gb</t>
+        </is>
+      </c>
+      <c r="H130" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="I130" s="3" t="inlineStr"/>
+      <c r="J130" s="2" t="inlineStr"/>
+      <c r="K130" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="L130" s="2" t="inlineStr">
+        <is>
+          <t>15 GB de franquia 31 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M130" s="2" t="inlineStr"/>
+      <c r="N130" s="2" t="inlineStr"/>
+      <c r="O130" s="2" t="inlineStr"/>
+      <c r="P130" s="2" t="inlineStr"/>
+      <c r="Q130" s="2" t="inlineStr"/>
+      <c r="R130" s="2" t="inlineStr">
+        <is>
+          <t>6 meses grátis de Gemini com AI Plus</t>
+        </is>
+      </c>
+      <c r="S130" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-controle</t>
+        </is>
+      </c>
+      <c r="T130" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E131" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F131" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Controle</t>
+        </is>
+      </c>
+      <c r="G131" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029300-61gb</t>
+        </is>
+      </c>
+      <c r="H131" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="I131" s="6" t="inlineStr"/>
+      <c r="J131" s="5" t="inlineStr"/>
+      <c r="K131" s="7" t="n">
+        <v>61</v>
+      </c>
+      <c r="L131" s="5" t="inlineStr">
+        <is>
+          <t>20 GB de franquia 31 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M131" s="5" t="inlineStr"/>
+      <c r="N131" s="5" t="inlineStr"/>
+      <c r="O131" s="5" t="inlineStr"/>
+      <c r="P131" s="5" t="inlineStr"/>
+      <c r="Q131" s="5" t="inlineStr"/>
+      <c r="R131" s="5" t="inlineStr">
+        <is>
+          <t>6 meses grátis de Gemini com AI Plus</t>
+        </is>
+      </c>
+      <c r="S131" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-controle</t>
+        </is>
+      </c>
+      <c r="T131" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle Educação</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029273-61gb</t>
+        </is>
+      </c>
+      <c r="H132" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="I132" s="3" t="inlineStr"/>
+      <c r="J132" s="2" t="inlineStr"/>
+      <c r="K132" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="L132" s="2" t="inlineStr">
+        <is>
+          <t>20 GB de franquia 31 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M132" s="2" t="inlineStr"/>
+      <c r="N132" s="2" t="inlineStr"/>
+      <c r="O132" s="2" t="inlineStr"/>
+      <c r="P132" s="2" t="inlineStr"/>
+      <c r="Q132" s="2" t="inlineStr"/>
+      <c r="R132" s="2" t="inlineStr">
+        <is>
+          <t>Assinatura Vivae inclusa</t>
+        </is>
+      </c>
+      <c r="S132" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-controle</t>
+        </is>
+      </c>
+      <c r="T132" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D133" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E133" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F133" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Controle Entretenimento</t>
+        </is>
+      </c>
+      <c r="G133" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029307-61gb</t>
+        </is>
+      </c>
+      <c r="H133" s="6" t="n">
+        <v>110</v>
+      </c>
+      <c r="I133" s="6" t="inlineStr"/>
+      <c r="J133" s="5" t="inlineStr"/>
+      <c r="K133" s="7" t="n">
+        <v>61</v>
+      </c>
+      <c r="L133" s="5" t="inlineStr">
+        <is>
+          <t>20 GB de franquia 31 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M133" s="5" t="inlineStr"/>
+      <c r="N133" s="5" t="inlineStr"/>
+      <c r="O133" s="5" t="inlineStr"/>
+      <c r="P133" s="5" t="inlineStr"/>
+      <c r="Q133" s="5" t="inlineStr"/>
+      <c r="R133" s="5" t="inlineStr">
+        <is>
+          <t>Assinatura Vivo TV Inicial inclusa</t>
+        </is>
+      </c>
+      <c r="S133" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-controle</t>
+        </is>
+      </c>
+      <c r="T133" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle Música</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029313-61gb</t>
+        </is>
+      </c>
+      <c r="H134" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="I134" s="3" t="inlineStr"/>
+      <c r="J134" s="2" t="inlineStr"/>
+      <c r="K134" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="L134" s="2" t="inlineStr">
+        <is>
+          <t>20 GB de franquia 31 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M134" s="2" t="inlineStr"/>
+      <c r="N134" s="2" t="inlineStr"/>
+      <c r="O134" s="2" t="inlineStr"/>
+      <c r="P134" s="2" t="inlineStr"/>
+      <c r="Q134" s="2" t="inlineStr"/>
+      <c r="R134" s="2" t="inlineStr">
+        <is>
+          <t>Apple Music Individual</t>
+        </is>
+      </c>
+      <c r="S134" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-controle</t>
+        </is>
+      </c>
+      <c r="T134" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D135" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E135" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F135" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Controle Netflix</t>
+        </is>
+      </c>
+      <c r="G135" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029308-61gb</t>
+        </is>
+      </c>
+      <c r="H135" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="I135" s="6" t="inlineStr"/>
+      <c r="J135" s="5" t="inlineStr"/>
+      <c r="K135" s="7" t="n">
+        <v>61</v>
+      </c>
+      <c r="L135" s="5" t="inlineStr">
+        <is>
+          <t>20 GB de franquia 31 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M135" s="5" t="inlineStr"/>
+      <c r="N135" s="5" t="inlineStr"/>
+      <c r="O135" s="5" t="inlineStr"/>
+      <c r="P135" s="5" t="inlineStr"/>
+      <c r="Q135" s="5" t="inlineStr"/>
+      <c r="R135" s="5" t="inlineStr">
+        <is>
+          <t>Assinatura Netflix Padrão com anúncios</t>
+        </is>
+      </c>
+      <c r="S135" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-controle</t>
+        </is>
+      </c>
+      <c r="T135" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle Saúde</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029301-61gb</t>
+        </is>
+      </c>
+      <c r="H136" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="I136" s="3" t="inlineStr"/>
+      <c r="J136" s="2" t="inlineStr"/>
+      <c r="K136" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="L136" s="2" t="inlineStr">
+        <is>
+          <t>20 GB de franquia 31 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M136" s="2" t="inlineStr"/>
+      <c r="N136" s="2" t="inlineStr"/>
+      <c r="O136" s="2" t="inlineStr"/>
+      <c r="P136" s="2" t="inlineStr"/>
+      <c r="Q136" s="2" t="inlineStr"/>
+      <c r="R136" s="2" t="inlineStr">
+        <is>
+          <t>Assinatura Vale Saúde Sempre inclusa</t>
+        </is>
+      </c>
+      <c r="S136" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-controle</t>
+        </is>
+      </c>
+      <c r="T136" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>lite</t>
+        </is>
+      </c>
+      <c r="E137" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F137" s="5" t="inlineStr">
+        <is>
+          <t>Easy Lite</t>
+        </is>
+      </c>
+      <c r="G137" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600025883-30gb</t>
+        </is>
+      </c>
+      <c r="H137" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I137" s="6" t="inlineStr"/>
+      <c r="J137" s="5" t="inlineStr"/>
+      <c r="K137" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="L137" s="5" t="inlineStr">
+        <is>
+          <t>30 GB de franquia</t>
+        </is>
+      </c>
+      <c r="M137" s="5" t="inlineStr"/>
+      <c r="N137" s="5" t="inlineStr"/>
+      <c r="O137" s="5" t="inlineStr"/>
+      <c r="P137" s="5" t="inlineStr"/>
+      <c r="Q137" s="5" t="inlineStr"/>
+      <c r="R137" s="5" t="inlineStr">
+        <is>
+          <t>2 meses de YouTube sem desconto no plano</t>
+        </is>
+      </c>
+      <c r="S137" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/easy-lite</t>
+        </is>
+      </c>
+      <c r="T137" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_lite_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>lite</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>Easy Lite</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600025885-40gb</t>
+        </is>
+      </c>
+      <c r="H138" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="I138" s="3" t="inlineStr"/>
+      <c r="J138" s="2" t="inlineStr"/>
+      <c r="K138" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="L138" s="2" t="inlineStr">
+        <is>
+          <t>40 GB de franquia</t>
+        </is>
+      </c>
+      <c r="M138" s="2" t="inlineStr"/>
+      <c r="N138" s="2" t="inlineStr"/>
+      <c r="O138" s="2" t="inlineStr"/>
+      <c r="P138" s="2" t="inlineStr"/>
+      <c r="Q138" s="2" t="inlineStr"/>
+      <c r="R138" s="2" t="inlineStr">
+        <is>
+          <t>2 meses de YouTube sem desconto no plano</t>
+        </is>
+      </c>
+      <c r="S138" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/easy-lite</t>
+        </is>
+      </c>
+      <c r="T138" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_lite_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t>lite</t>
+        </is>
+      </c>
+      <c r="E139" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F139" s="5" t="inlineStr">
+        <is>
+          <t>Easy Lite</t>
+        </is>
+      </c>
+      <c r="G139" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600025888-20gb</t>
+        </is>
+      </c>
+      <c r="H139" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="I139" s="6" t="inlineStr"/>
+      <c r="J139" s="5" t="inlineStr"/>
+      <c r="K139" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="L139" s="5" t="inlineStr">
+        <is>
+          <t>20 GB de franquia</t>
+        </is>
+      </c>
+      <c r="M139" s="5" t="inlineStr"/>
+      <c r="N139" s="5" t="inlineStr"/>
+      <c r="O139" s="5" t="inlineStr"/>
+      <c r="P139" s="5" t="inlineStr"/>
+      <c r="Q139" s="5" t="inlineStr"/>
+      <c r="R139" s="5" t="inlineStr">
+        <is>
+          <t>2 meses de YouTube sem desconto no plano</t>
+        </is>
+      </c>
+      <c r="S139" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/easy-lite</t>
+        </is>
+      </c>
+      <c r="T139" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_lite_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Pós com Amazon</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029255-60gb</t>
+        </is>
+      </c>
+      <c r="H140" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="I140" s="3" t="inlineStr"/>
+      <c r="J140" s="2" t="inlineStr"/>
+      <c r="K140" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="L140" s="2" t="inlineStr">
+        <is>
+          <t>50 GB de franquia 10 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M140" s="2" t="inlineStr"/>
+      <c r="N140" s="2" t="inlineStr"/>
+      <c r="O140" s="2" t="inlineStr"/>
+      <c r="P140" s="2" t="inlineStr"/>
+      <c r="Q140" s="2" t="inlineStr"/>
+      <c r="R140" s="2" t="inlineStr">
+        <is>
+          <t>Assinatura Amazon Prime inclusa</t>
+        </is>
+      </c>
+      <c r="S140" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-pos-pago</t>
+        </is>
+      </c>
+      <c r="T140" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D141" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E141" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F141" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Pós com Disney+</t>
+        </is>
+      </c>
+      <c r="G141" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600022115-60gb</t>
+        </is>
+      </c>
+      <c r="H141" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="I141" s="6" t="inlineStr"/>
+      <c r="J141" s="5" t="inlineStr"/>
+      <c r="K141" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="L141" s="5" t="inlineStr">
+        <is>
+          <t>50 GB de franquia 10 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M141" s="5" t="inlineStr"/>
+      <c r="N141" s="5" t="inlineStr"/>
+      <c r="O141" s="5" t="inlineStr"/>
+      <c r="P141" s="5" t="inlineStr">
+        <is>
+          <t>Disney+</t>
+        </is>
+      </c>
+      <c r="Q141" s="5" t="inlineStr"/>
+      <c r="R141" s="5" t="inlineStr">
+        <is>
+          <t>Assinatura Disney+ Padrão inclusa</t>
+        </is>
+      </c>
+      <c r="S141" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-pos-pago</t>
+        </is>
+      </c>
+      <c r="T141" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Pós com Globoplay</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029246-60gb</t>
+        </is>
+      </c>
+      <c r="H142" s="3" t="n">
+        <v>165</v>
+      </c>
+      <c r="I142" s="3" t="inlineStr"/>
+      <c r="J142" s="2" t="inlineStr"/>
+      <c r="K142" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="L142" s="2" t="inlineStr">
+        <is>
+          <t>50 GB de franquia 10 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M142" s="2" t="inlineStr"/>
+      <c r="N142" s="2" t="inlineStr"/>
+      <c r="O142" s="2" t="inlineStr"/>
+      <c r="P142" s="2" t="inlineStr">
+        <is>
+          <t>Globoplay</t>
+        </is>
+      </c>
+      <c r="Q142" s="2" t="inlineStr"/>
+      <c r="R142" s="2" t="inlineStr">
+        <is>
+          <t>Assinatura Globoplay inclusa</t>
+        </is>
+      </c>
+      <c r="S142" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-pos-pago</t>
+        </is>
+      </c>
+      <c r="T142" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F143" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Pós com Netflix</t>
+        </is>
+      </c>
+      <c r="G143" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029234-60gb</t>
+        </is>
+      </c>
+      <c r="H143" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="I143" s="6" t="inlineStr"/>
+      <c r="J143" s="5" t="inlineStr"/>
+      <c r="K143" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="L143" s="5" t="inlineStr">
+        <is>
+          <t>50 GB de franquia 10 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M143" s="5" t="inlineStr"/>
+      <c r="N143" s="5" t="inlineStr"/>
+      <c r="O143" s="5" t="inlineStr"/>
+      <c r="P143" s="5" t="inlineStr">
+        <is>
+          <t>Netflix</t>
+        </is>
+      </c>
+      <c r="Q143" s="5" t="inlineStr"/>
+      <c r="R143" s="5" t="inlineStr">
+        <is>
+          <t>Assinatura Netflix Padrão inclusa</t>
+        </is>
+      </c>
+      <c r="S143" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-pos-pago</t>
+        </is>
+      </c>
+      <c r="T143" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Pós com Premiere</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029249-60gb</t>
+        </is>
+      </c>
+      <c r="H144" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="I144" s="3" t="inlineStr"/>
+      <c r="J144" s="2" t="inlineStr"/>
+      <c r="K144" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="L144" s="2" t="inlineStr">
+        <is>
+          <t>50 GB de franquia 10 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M144" s="2" t="inlineStr"/>
+      <c r="N144" s="2" t="inlineStr"/>
+      <c r="O144" s="2" t="inlineStr"/>
+      <c r="P144" s="2" t="inlineStr">
+        <is>
+          <t>Premiere</t>
+        </is>
+      </c>
+      <c r="Q144" s="2" t="inlineStr"/>
+      <c r="R144" s="2" t="inlineStr">
+        <is>
+          <t>Assinatura Premiere inclusa</t>
+        </is>
+      </c>
+      <c r="S144" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-pos-pago</t>
+        </is>
+      </c>
+      <c r="T144" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E145" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F145" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Pós com Spotify</t>
+        </is>
+      </c>
+      <c r="G145" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029229-60gb</t>
+        </is>
+      </c>
+      <c r="H145" s="6" t="n">
+        <v>165</v>
+      </c>
+      <c r="I145" s="6" t="inlineStr"/>
+      <c r="J145" s="5" t="inlineStr"/>
+      <c r="K145" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="L145" s="5" t="inlineStr">
+        <is>
+          <t>50 GB de franquia 10 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M145" s="5" t="inlineStr"/>
+      <c r="N145" s="5" t="inlineStr"/>
+      <c r="O145" s="5" t="inlineStr"/>
+      <c r="P145" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="Q145" s="5" t="inlineStr"/>
+      <c r="R145" s="5" t="inlineStr">
+        <is>
+          <t>Assinatura Spotify Premium inclusa</t>
+        </is>
+      </c>
+      <c r="S145" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-pos-pago</t>
+        </is>
+      </c>
+      <c r="T145" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Pós com Travel</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029244-70gb</t>
+        </is>
+      </c>
+      <c r="H146" s="3" t="n">
+        <v>215</v>
+      </c>
+      <c r="I146" s="3" t="inlineStr"/>
+      <c r="J146" s="2" t="inlineStr"/>
+      <c r="K146" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="L146" s="2" t="inlineStr">
+        <is>
+          <t>60 GB de franquia 10 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M146" s="2" t="inlineStr"/>
+      <c r="N146" s="2" t="inlineStr"/>
+      <c r="O146" s="2" t="inlineStr"/>
+      <c r="P146" s="2" t="inlineStr"/>
+      <c r="Q146" s="2" t="inlineStr"/>
+      <c r="R146" s="2" t="inlineStr">
+        <is>
+          <t>6 meses grátis de Gemini com AI Plus</t>
+        </is>
+      </c>
+      <c r="S146" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-pos-pago</t>
+        </is>
+      </c>
+      <c r="T146" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F147" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Pré</t>
+        </is>
+      </c>
+      <c r="G147" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600022379-25gb</t>
+        </is>
+      </c>
+      <c r="H147" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I147" s="6" t="inlineStr"/>
+      <c r="J147" s="5" t="inlineStr"/>
+      <c r="K147" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="L147" s="5" t="inlineStr">
+        <is>
+          <t>15 GB para navegar como quiser 5 GB de bônus 5 GB para navegar no Youtube</t>
+        </is>
+      </c>
+      <c r="M147" s="5" t="inlineStr"/>
+      <c r="N147" s="5" t="inlineStr"/>
+      <c r="O147" s="5" t="inlineStr"/>
+      <c r="P147" s="5" t="inlineStr"/>
+      <c r="Q147" s="5" t="inlineStr"/>
+      <c r="R147" s="5" t="inlineStr"/>
+      <c r="S147" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/pre-pago/vivo-pre</t>
+        </is>
+      </c>
+      <c r="T147" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_prepaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Pré</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600022379-9gb</t>
+        </is>
+      </c>
+      <c r="H148" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="I148" s="3" t="inlineStr"/>
+      <c r="J148" s="2" t="inlineStr"/>
+      <c r="K148" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="L148" s="2" t="inlineStr">
+        <is>
+          <t>6 GB para navegar como quiser 3 GB para navegar no YouTube</t>
+        </is>
+      </c>
+      <c r="M148" s="2" t="inlineStr"/>
+      <c r="N148" s="2" t="inlineStr"/>
+      <c r="O148" s="2" t="inlineStr"/>
+      <c r="P148" s="2" t="inlineStr"/>
+      <c r="Q148" s="2" t="inlineStr"/>
+      <c r="R148" s="2" t="inlineStr"/>
+      <c r="S148" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/pre-pago/vivo-pre</t>
+        </is>
+      </c>
+      <c r="T148" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_prepaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F149" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Pré</t>
+        </is>
+      </c>
+      <c r="G149" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600022379-5gb</t>
+        </is>
+      </c>
+      <c r="H149" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="I149" s="6" t="inlineStr"/>
+      <c r="J149" s="5" t="inlineStr"/>
+      <c r="K149" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L149" s="5" t="inlineStr">
+        <is>
+          <t>5 GB para navegar como quiser</t>
+        </is>
+      </c>
+      <c r="M149" s="5" t="inlineStr"/>
+      <c r="N149" s="5" t="inlineStr"/>
+      <c r="O149" s="5" t="inlineStr"/>
+      <c r="P149" s="5" t="inlineStr"/>
+      <c r="Q149" s="5" t="inlineStr"/>
+      <c r="R149" s="5" t="inlineStr"/>
+      <c r="S149" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/pre-pago/vivo-pre</t>
+        </is>
+      </c>
+      <c r="T149" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_prepaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T22:14:36</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Pré</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600022379-4gb</t>
+        </is>
+      </c>
+      <c r="H150" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="I150" s="3" t="inlineStr"/>
+      <c r="J150" s="2" t="inlineStr"/>
+      <c r="K150" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L150" s="2" t="inlineStr">
+        <is>
+          <t>4 GB para navegar como quiser</t>
+        </is>
+      </c>
+      <c r="M150" s="2" t="inlineStr"/>
+      <c r="N150" s="2" t="inlineStr"/>
+      <c r="O150" s="2" t="inlineStr"/>
+      <c r="P150" s="2" t="inlineStr"/>
+      <c r="Q150" s="2" t="inlineStr"/>
+      <c r="R150" s="2" t="inlineStr"/>
+      <c r="S150" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/pre-pago/vivo-pre</t>
+        </is>
+      </c>
+      <c r="T150" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_prepaid_SP.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T101"/>
+  <autoFilter ref="A1:T150"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8429,12 +11743,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -8505,12 +11819,12 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -8575,12 +11889,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -8645,12 +11959,12 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -8715,12 +12029,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -8785,12 +12099,12 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -8855,12 +12169,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -8925,12 +12239,12 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -8995,12 +12309,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -9065,12 +12379,12 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -9135,12 +12449,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -9205,12 +12519,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -9275,12 +12589,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -9341,12 +12655,12 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -9403,12 +12717,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -9465,12 +12779,12 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -9527,12 +12841,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -9589,12 +12903,12 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -9649,12 +12963,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -9711,12 +13025,12 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -9773,12 +13087,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -9835,12 +13149,12 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -9897,12 +13211,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -9959,12 +13273,12 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -10021,12 +13335,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -10083,12 +13397,12 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -10145,12 +13459,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -10207,12 +13521,12 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -10269,12 +13583,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -10339,12 +13653,12 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -10409,12 +13723,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -10479,12 +13793,12 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -10549,12 +13863,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -10619,12 +13933,12 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -10689,12 +14003,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -10759,12 +14073,12 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -10789,7 +14103,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600005312-30gb</t>
+          <t>vivo:VIV202600025883-30gb</t>
         </is>
       </c>
       <c r="H37" s="6" t="n">
@@ -10812,7 +14126,7 @@
       <c r="Q37" s="5" t="inlineStr"/>
       <c r="R37" s="5" t="inlineStr">
         <is>
-          <t>Youtube Ilimitado</t>
+          <t>2 meses de YouTube sem desconto no plano</t>
         </is>
       </c>
       <c r="S37" s="5" t="inlineStr">
@@ -10829,12 +14143,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -10859,7 +14173,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600019134-40gb</t>
+          <t>vivo:VIV202600025885-40gb</t>
         </is>
       </c>
       <c r="H38" s="3" t="n">
@@ -10882,7 +14196,7 @@
       <c r="Q38" s="2" t="inlineStr"/>
       <c r="R38" s="2" t="inlineStr">
         <is>
-          <t>Youtube Ilimitado</t>
+          <t>2 meses de YouTube sem desconto no plano</t>
         </is>
       </c>
       <c r="S38" s="2" t="inlineStr">
@@ -10899,12 +14213,12 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -10929,7 +14243,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600019132-20gb</t>
+          <t>vivo:VIV202600025888-20gb</t>
         </is>
       </c>
       <c r="H39" s="6" t="n">
@@ -10952,7 +14266,7 @@
       <c r="Q39" s="5" t="inlineStr"/>
       <c r="R39" s="5" t="inlineStr">
         <is>
-          <t>Youtube Ilimitado</t>
+          <t>2 meses de YouTube sem desconto no plano</t>
         </is>
       </c>
       <c r="S39" s="5" t="inlineStr">
@@ -10969,12 +14283,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -11039,12 +14353,12 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -11113,12 +14427,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -11187,12 +14501,12 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -11261,12 +14575,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -11335,12 +14649,12 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -11409,12 +14723,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -11479,12 +14793,12 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -11545,12 +14859,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -11611,12 +14925,12 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -11677,12 +14991,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -11770,7 +15084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11834,7 +15148,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>removed</t>
+          <t>new</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -11854,7 +15168,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600019127-30gb</t>
+          <t>vivo:VIV202600025883-30gb</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -11862,48 +15176,196 @@
           <t>Easy Lite</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H2" s="3" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr"/>
+      <c r="H2" s="3" t="n">
+        <v>30</v>
+      </c>
       <c r="I2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>lite</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600025885-40gb</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Easy Lite</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr"/>
+      <c r="H3" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="I3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>lite</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600025888-20gb</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Easy Lite</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="I4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
           <t>removed</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>vivo</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>lite</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>vivo:VIV202600019129-40gb</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600005312-30gb</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Easy Lite</t>
         </is>
       </c>
-      <c r="G3" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="H3" s="6" t="inlineStr"/>
-      <c r="I3" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>lite</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600019132-20gb</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Easy Lite</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>lite</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600019134-40gb</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Easy Lite</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11942,7 +15404,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T22:10:23</t>
+          <t>2026-06-24T22:14:36</t>
         </is>
       </c>
     </row>
@@ -11954,7 +15416,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
     </row>
@@ -11975,7 +15437,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -12086,7 +15548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -12319,8 +15781,63 @@
         <v/>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="12" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B39" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"control",history!$A:$A,$A39)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"control",history!$A:$A,$A39))</f>
+        <v/>
+      </c>
+      <c r="C39" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"control",history!$A:$A,$A39)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"control",history!$A:$A,$A39))</f>
+        <v/>
+      </c>
+      <c r="D39" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"control",history!$A:$A,$A39)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"control",history!$A:$A,$A39))</f>
+        <v/>
+      </c>
+      <c r="E39" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"postpaid",history!$A:$A,$A39)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"postpaid",history!$A:$A,$A39))</f>
+        <v/>
+      </c>
+      <c r="F39" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"postpaid",history!$A:$A,$A39)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"postpaid",history!$A:$A,$A39))</f>
+        <v/>
+      </c>
+      <c r="G39" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"postpaid",history!$A:$A,$A39)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"postpaid",history!$A:$A,$A39))</f>
+        <v/>
+      </c>
+      <c r="H39" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"prepaid",history!$A:$A,$A39)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"prepaid",history!$A:$A,$A39))</f>
+        <v/>
+      </c>
+      <c r="I39" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"prepaid",history!$A:$A,$A39)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"prepaid",history!$A:$A,$A39))</f>
+        <v/>
+      </c>
+      <c r="J39" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"prepaid",history!$A:$A,$A39)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"prepaid",history!$A:$A,$A39))</f>
+        <v/>
+      </c>
+      <c r="K39" s="3">
+        <f>IFERROR(1/MAX(IFERROR(1/_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"lite",history!$A:$A,$A39),0),IFERROR(1/_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"flex",history!$A:$A,$A39),0)),"")</f>
+        <v/>
+      </c>
+      <c r="L39" s="3">
+        <f>IFERROR(1/MAX(IFERROR(1/_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"lite",history!$A:$A,$A39),0),IFERROR(1/_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"flex",history!$A:$A,$A39),0)),"")</f>
+        <v/>
+      </c>
+      <c r="M39" s="3">
+        <f>IFERROR(1/MAX(IFERROR(1/_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"lite",history!$A:$A,$A39),0),IFERROR(1/_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"flex",history!$A:$A,$A39),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t>Pre = cheapest recharge amount captured (true R$/day needs validity-days we don't yet capture — CONTEXT §8). Digital = min of Vivo Lite / Claro Flex. Daily rows now; monthly roll-up is the planned next step.</t>
         </is>
@@ -12334,7 +15851,7 @@
     <mergeCell ref="K35:M35"/>
     <mergeCell ref="H35:J35"/>
   </mergeCells>
-  <conditionalFormatting sqref="B37:D38">
+  <conditionalFormatting sqref="B37:D39">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -12346,7 +15863,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E37:G38">
+  <conditionalFormatting sqref="E37:G39">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -12358,7 +15875,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H37:J38">
+  <conditionalFormatting sqref="H37:J39">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -12370,7 +15887,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K37:M38">
+  <conditionalFormatting sqref="K37:M39">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -13670,7 +17187,7 @@
       <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Youtube Ilimitado</t>
+          <t>2 meses de YouTube sem desconto no plano</t>
         </is>
       </c>
     </row>
@@ -13694,7 +17211,7 @@
       <c r="G20" s="5" t="n"/>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Youtube Ilimitado</t>
+          <t>2 meses de YouTube sem desconto no plano</t>
         </is>
       </c>
     </row>
@@ -13718,7 +17235,7 @@
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Youtube Ilimitado</t>
+          <t>2 meses de YouTube sem desconto no plano</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): daily snapshot 2026-06-25
</commit_message>
<xml_diff>
--- a/projects/mobile-price-tracker/data/mobile_plans.xlsx
+++ b/projects/mobile-price-tracker/data/mobile_plans.xlsx
@@ -18,7 +18,7 @@
     <sheet name="TIM" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'history'!$A$1:$T$150</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'history'!$A$1:$T$199</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'latest'!$A$1:$T$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -296,12 +296,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$39</f>
+              <f>'comparison'!$A$37:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$B$37:$B$39</f>
+              <f>'comparison'!$B$37:$B$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -333,12 +333,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$39</f>
+              <f>'comparison'!$A$37:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$C$37:$C$39</f>
+              <f>'comparison'!$C$37:$C$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -370,12 +370,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$39</f>
+              <f>'comparison'!$A$37:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$D$37:$D$39</f>
+              <f>'comparison'!$D$37:$D$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -493,12 +493,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$39</f>
+              <f>'comparison'!$A$37:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$E$37:$E$39</f>
+              <f>'comparison'!$E$37:$E$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -530,12 +530,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$39</f>
+              <f>'comparison'!$A$37:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$F$37:$F$39</f>
+              <f>'comparison'!$F$37:$F$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -567,12 +567,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$39</f>
+              <f>'comparison'!$A$37:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$G$37:$G$39</f>
+              <f>'comparison'!$G$37:$G$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -690,12 +690,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$39</f>
+              <f>'comparison'!$A$37:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$H$37:$H$39</f>
+              <f>'comparison'!$H$37:$H$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -727,12 +727,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$39</f>
+              <f>'comparison'!$A$37:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$I$37:$I$39</f>
+              <f>'comparison'!$I$37:$I$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -764,12 +764,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$39</f>
+              <f>'comparison'!$A$37:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$J$37:$J$39</f>
+              <f>'comparison'!$J$37:$J$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -887,12 +887,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$39</f>
+              <f>'comparison'!$A$37:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$K$37:$K$39</f>
+              <f>'comparison'!$K$37:$K$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -924,12 +924,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$39</f>
+              <f>'comparison'!$A$37:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$L$37:$L$39</f>
+              <f>'comparison'!$L$37:$L$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -961,12 +961,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'comparison'!$A$37:$A$39</f>
+              <f>'comparison'!$A$37:$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'comparison'!$M$37:$M$39</f>
+              <f>'comparison'!$M$37:$M$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1419,7 +1419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T150"/>
+  <dimension ref="A1:T199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -11600,8 +11600,3322 @@
         </is>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E151" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F151" s="5" t="inlineStr">
+        <is>
+          <t>Controle 25GB</t>
+        </is>
+      </c>
+      <c r="G151" s="5" t="inlineStr">
+        <is>
+          <t>claro:plano-controle-25gb</t>
+        </is>
+      </c>
+      <c r="H151" s="6" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="I151" s="6" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="J151" s="5" t="inlineStr">
+        <is>
+          <t>De R$ 59,90 Por:</t>
+        </is>
+      </c>
+      <c r="K151" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="L151" s="5" t="inlineStr"/>
+      <c r="M151" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N151" s="5" t="inlineStr"/>
+      <c r="O151" s="5" t="inlineStr"/>
+      <c r="P151" s="5" t="inlineStr"/>
+      <c r="Q151" s="5" t="inlineStr"/>
+      <c r="R151" s="5" t="inlineStr">
+        <is>
+          <t>Para uso livre; Para redes sociais e vídeos; Bônus exclusivo; Aproveite na sua franquia; WhatsApp e ligações ilimitadas</t>
+        </is>
+      </c>
+      <c r="S151" s="5" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/controle</t>
+        </is>
+      </c>
+      <c r="T151" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/claro_control_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>Controle 30GB</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>claro:plano-controle-30gb</t>
+        </is>
+      </c>
+      <c r="H152" s="3" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="I152" s="3" t="inlineStr"/>
+      <c r="J152" s="2" t="inlineStr"/>
+      <c r="K152" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="L152" s="2" t="inlineStr"/>
+      <c r="M152" s="2" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N152" s="2" t="inlineStr"/>
+      <c r="O152" s="2" t="inlineStr"/>
+      <c r="P152" s="2" t="inlineStr"/>
+      <c r="Q152" s="2" t="inlineStr"/>
+      <c r="R152" s="2" t="inlineStr">
+        <is>
+          <t>Para uso livre; Bônus do Hexa para uso livre; Bônus para redes sociais e apps; Redes sociais e apps; WhatsApp ilimitado</t>
+        </is>
+      </c>
+      <c r="S152" s="2" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/controle</t>
+        </is>
+      </c>
+      <c r="T152" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/claro_control_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F153" s="5" t="inlineStr">
+        <is>
+          <t>Controle 30GB</t>
+        </is>
+      </c>
+      <c r="G153" s="5" t="inlineStr">
+        <is>
+          <t>claro:plano-controle-30gb-gaming</t>
+        </is>
+      </c>
+      <c r="H153" s="6" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="I153" s="6" t="inlineStr"/>
+      <c r="J153" s="5" t="inlineStr"/>
+      <c r="K153" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="L153" s="5" t="inlineStr"/>
+      <c r="M153" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N153" s="5" t="inlineStr"/>
+      <c r="O153" s="5" t="inlineStr"/>
+      <c r="P153" s="5" t="inlineStr"/>
+      <c r="Q153" s="5" t="inlineStr"/>
+      <c r="R153" s="5" t="inlineStr">
+        <is>
+          <t>Para uso livre; Bônus para redes sociais e apps; Bônus uso livre; Redes sociais e apps; WhatsApp ilimitado</t>
+        </is>
+      </c>
+      <c r="S153" s="5" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/controle</t>
+        </is>
+      </c>
+      <c r="T153" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/claro_control_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>flex</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>Flex 15GB</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>claro:plano-flex-15gb</t>
+        </is>
+      </c>
+      <c r="H154" s="3" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="I154" s="3" t="inlineStr"/>
+      <c r="J154" s="2" t="inlineStr"/>
+      <c r="K154" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="L154" s="2" t="inlineStr"/>
+      <c r="M154" s="2" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N154" s="2" t="inlineStr"/>
+      <c r="O154" s="2" t="inlineStr"/>
+      <c r="P154" s="2" t="inlineStr"/>
+      <c r="Q154" s="2" t="inlineStr"/>
+      <c r="R154" s="2" t="inlineStr">
+        <is>
+          <t>Para uso livre; Bônus do Hexa para uso livre; Para redes sociais e apps; Bônus extra nos apps; WhatsApp ilimitado</t>
+        </is>
+      </c>
+      <c r="S154" s="2" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/flex</t>
+        </is>
+      </c>
+      <c r="T154" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/claro_flex_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>flex</t>
+        </is>
+      </c>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F155" s="5" t="inlineStr">
+        <is>
+          <t>Flex 20GB</t>
+        </is>
+      </c>
+      <c r="G155" s="5" t="inlineStr">
+        <is>
+          <t>claro:plano-flex-20gb</t>
+        </is>
+      </c>
+      <c r="H155" s="6" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="I155" s="6" t="inlineStr"/>
+      <c r="J155" s="5" t="inlineStr"/>
+      <c r="K155" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="L155" s="5" t="inlineStr"/>
+      <c r="M155" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N155" s="5" t="inlineStr"/>
+      <c r="O155" s="5" t="inlineStr"/>
+      <c r="P155" s="5" t="inlineStr"/>
+      <c r="Q155" s="5" t="inlineStr"/>
+      <c r="R155" s="5" t="inlineStr">
+        <is>
+          <t>Para uso livre; Bônus do Hexa para uso livre; Para redes sociais e apps; Bônus extra nos apps; WhatsApp ilimitado</t>
+        </is>
+      </c>
+      <c r="S155" s="5" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/flex</t>
+        </is>
+      </c>
+      <c r="T155" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/claro_flex_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>flex</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>Flex 30GB</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>claro:plano-flex-30gb</t>
+        </is>
+      </c>
+      <c r="H156" s="3" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="I156" s="3" t="inlineStr"/>
+      <c r="J156" s="2" t="inlineStr"/>
+      <c r="K156" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="L156" s="2" t="inlineStr"/>
+      <c r="M156" s="2" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N156" s="2" t="inlineStr"/>
+      <c r="O156" s="2" t="inlineStr"/>
+      <c r="P156" s="2" t="inlineStr"/>
+      <c r="Q156" s="2" t="inlineStr"/>
+      <c r="R156" s="2" t="inlineStr">
+        <is>
+          <t>Para uso livre; Bônus do Hexa para uso livre; Para redes sociais e apps; Bônus extra nos apps; WhatsApp ilimitado; Assinatura Claro musica inclusa</t>
+        </is>
+      </c>
+      <c r="S156" s="2" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/flex</t>
+        </is>
+      </c>
+      <c r="T156" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/claro_flex_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>flex</t>
+        </is>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F157" s="5" t="inlineStr">
+        <is>
+          <t>Flex 40GB</t>
+        </is>
+      </c>
+      <c r="G157" s="5" t="inlineStr">
+        <is>
+          <t>claro:plano-flex-40gb</t>
+        </is>
+      </c>
+      <c r="H157" s="6" t="n">
+        <v>119.9</v>
+      </c>
+      <c r="I157" s="6" t="inlineStr"/>
+      <c r="J157" s="5" t="inlineStr"/>
+      <c r="K157" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="L157" s="5" t="inlineStr"/>
+      <c r="M157" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N157" s="5" t="inlineStr"/>
+      <c r="O157" s="5" t="inlineStr"/>
+      <c r="P157" s="5" t="inlineStr"/>
+      <c r="Q157" s="5" t="inlineStr"/>
+      <c r="R157" s="5" t="inlineStr">
+        <is>
+          <t>Para uso livre; Para redes sociais e apps; Bônus uso livre; Bônus extra nos apps; WhatsApp ilimitado; Assinatura Claro musica inclusa</t>
+        </is>
+      </c>
+      <c r="S157" s="5" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/flex</t>
+        </is>
+      </c>
+      <c r="T157" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/claro_flex_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>Pós 100GB</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="inlineStr">
+        <is>
+          <t>claro:plano-pos-100gb</t>
+        </is>
+      </c>
+      <c r="H158" s="3" t="n">
+        <v>179.9</v>
+      </c>
+      <c r="I158" s="3" t="inlineStr"/>
+      <c r="J158" s="2" t="inlineStr"/>
+      <c r="K158" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="L158" s="2" t="inlineStr"/>
+      <c r="M158" s="2" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N158" s="2" t="inlineStr"/>
+      <c r="O158" s="2" t="inlineStr"/>
+      <c r="P158" s="2" t="inlineStr"/>
+      <c r="Q158" s="2" t="inlineStr"/>
+      <c r="R158" s="2" t="inlineStr">
+        <is>
+          <t>Armazenamento na nuvem:; Google One ou iCloud+; WhatsApp ilimitado; Roaming: Passaporte Américas; Claro Sync: Smartwatch conectado</t>
+        </is>
+      </c>
+      <c r="S158" s="2" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/pos</t>
+        </is>
+      </c>
+      <c r="T158" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/claro_postpaid_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F159" s="5" t="inlineStr">
+        <is>
+          <t>Pós 150GB</t>
+        </is>
+      </c>
+      <c r="G159" s="5" t="inlineStr">
+        <is>
+          <t>claro:plano-pos-150gb</t>
+        </is>
+      </c>
+      <c r="H159" s="6" t="n">
+        <v>239.9</v>
+      </c>
+      <c r="I159" s="6" t="inlineStr"/>
+      <c r="J159" s="5" t="inlineStr"/>
+      <c r="K159" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="L159" s="5" t="inlineStr"/>
+      <c r="M159" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N159" s="5" t="inlineStr"/>
+      <c r="O159" s="5" t="inlineStr"/>
+      <c r="P159" s="5" t="inlineStr"/>
+      <c r="Q159" s="5" t="inlineStr"/>
+      <c r="R159" s="5" t="inlineStr">
+        <is>
+          <t>Armazenamento na nuvem:; Google One ou iCloud+; WhatsApp ilimitado; Roaming: Passaporte Américas e Europa; Claro Sync: Smartwatch conectado</t>
+        </is>
+      </c>
+      <c r="S159" s="5" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/pos</t>
+        </is>
+      </c>
+      <c r="T159" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/claro_postpaid_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>Pós 200GB</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>claro:plano-pos-200gb</t>
+        </is>
+      </c>
+      <c r="H160" s="3" t="n">
+        <v>339.9</v>
+      </c>
+      <c r="I160" s="3" t="inlineStr"/>
+      <c r="J160" s="2" t="inlineStr"/>
+      <c r="K160" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="L160" s="2" t="inlineStr"/>
+      <c r="M160" s="2" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N160" s="2" t="inlineStr"/>
+      <c r="O160" s="2" t="inlineStr"/>
+      <c r="P160" s="2" t="inlineStr"/>
+      <c r="Q160" s="2" t="inlineStr"/>
+      <c r="R160" s="2" t="inlineStr">
+        <is>
+          <t>Armazenamento na nuvem:; Google One ou iCloud+; WhatsApp ilimitado; Roaming: Passaporte Mundo; Claro Sync: Smartwatch conectado</t>
+        </is>
+      </c>
+      <c r="S160" s="2" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/pos</t>
+        </is>
+      </c>
+      <c r="T160" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/claro_postpaid_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F161" s="5" t="inlineStr">
+        <is>
+          <t>Pós 50GB com GeForce NOW</t>
+        </is>
+      </c>
+      <c r="G161" s="5" t="inlineStr">
+        <is>
+          <t>claro:plano-pos-60gb-geforce</t>
+        </is>
+      </c>
+      <c r="H161" s="6" t="n">
+        <v>164.9</v>
+      </c>
+      <c r="I161" s="6" t="inlineStr"/>
+      <c r="J161" s="5" t="inlineStr"/>
+      <c r="K161" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="L161" s="5" t="inlineStr"/>
+      <c r="M161" s="5" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N161" s="5" t="inlineStr"/>
+      <c r="O161" s="5" t="inlineStr"/>
+      <c r="P161" s="5" t="inlineStr"/>
+      <c r="Q161" s="5" t="inlineStr"/>
+      <c r="R161" s="5" t="inlineStr">
+        <is>
+          <t>Armazenamento na nuvem:; Google One ou iCloud+; WhatsApp ilimitado; Roaming: Passaporte Américas; Claro Sync: Smartwatch conectado; Inclusa assinatura GeForce NOW</t>
+        </is>
+      </c>
+      <c r="S161" s="5" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/pos</t>
+        </is>
+      </c>
+      <c r="T161" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/claro_postpaid_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>Pós 60GB</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>claro:plano-pos-60gb</t>
+        </is>
+      </c>
+      <c r="H162" s="3" t="n">
+        <v>124.9</v>
+      </c>
+      <c r="I162" s="3" t="inlineStr"/>
+      <c r="J162" s="2" t="inlineStr"/>
+      <c r="K162" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="L162" s="2" t="inlineStr"/>
+      <c r="M162" s="2" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="N162" s="2" t="inlineStr"/>
+      <c r="O162" s="2" t="inlineStr"/>
+      <c r="P162" s="2" t="inlineStr"/>
+      <c r="Q162" s="2" t="inlineStr"/>
+      <c r="R162" s="2" t="inlineStr">
+        <is>
+          <t>Armazenamento na nuvem:; Google One ou iCloud+; WhatsApp ilimitado; Roaming: Passaporte Américas; Claro Sync: Smartwatch conectado</t>
+        </is>
+      </c>
+      <c r="S162" s="2" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/pos</t>
+        </is>
+      </c>
+      <c r="T162" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/claro_postpaid_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F163" s="5" t="inlineStr">
+        <is>
+          <t>Prezão R$1 por dia</t>
+        </is>
+      </c>
+      <c r="G163" s="5" t="inlineStr">
+        <is>
+          <t>claro:prez-o-r-1-por-dia</t>
+        </is>
+      </c>
+      <c r="H163" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I163" s="6" t="inlineStr"/>
+      <c r="J163" s="5" t="inlineStr">
+        <is>
+          <t>prepaid Prezão — preço por dia; recargas a partir de R$15</t>
+        </is>
+      </c>
+      <c r="K163" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="L163" s="5" t="inlineStr"/>
+      <c r="M163" s="5" t="inlineStr"/>
+      <c r="N163" s="5" t="inlineStr"/>
+      <c r="O163" s="5" t="inlineStr"/>
+      <c r="P163" s="5" t="inlineStr"/>
+      <c r="Q163" s="5" t="inlineStr"/>
+      <c r="R163" s="5" t="inlineStr"/>
+      <c r="S163" s="5" t="inlineStr">
+        <is>
+          <t>https://www.claro.com.br/celular/planos-pre/prezao</t>
+        </is>
+      </c>
+      <c r="T163" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/claro_prepaid_SP.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>TIM Controle 41GB</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>tim:162901</t>
+        </is>
+      </c>
+      <c r="H164" s="3" t="n">
+        <v>58.99</v>
+      </c>
+      <c r="I164" s="3" t="inlineStr"/>
+      <c r="J164" s="2" t="inlineStr"/>
+      <c r="K164" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="L164" s="2" t="inlineStr"/>
+      <c r="M164" s="2" t="inlineStr"/>
+      <c r="N164" s="2" t="inlineStr"/>
+      <c r="O164" s="2" t="inlineStr"/>
+      <c r="P164" s="2" t="inlineStr"/>
+      <c r="Q164" s="2" t="inlineStr"/>
+      <c r="R164" s="2" t="inlineStr"/>
+      <c r="S164" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/controle</t>
+        </is>
+      </c>
+      <c r="T164" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D165" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E165" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F165" s="5" t="inlineStr">
+        <is>
+          <t>TIM Controle Light Express 31GB</t>
+        </is>
+      </c>
+      <c r="G165" s="5" t="inlineStr">
+        <is>
+          <t>tim:143536</t>
+        </is>
+      </c>
+      <c r="H165" s="6" t="n">
+        <v>60.99</v>
+      </c>
+      <c r="I165" s="6" t="inlineStr"/>
+      <c r="J165" s="5" t="inlineStr"/>
+      <c r="K165" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="L165" s="5" t="inlineStr"/>
+      <c r="M165" s="5" t="inlineStr"/>
+      <c r="N165" s="5" t="inlineStr"/>
+      <c r="O165" s="5" t="inlineStr"/>
+      <c r="P165" s="5" t="inlineStr"/>
+      <c r="Q165" s="5" t="inlineStr"/>
+      <c r="R165" s="5" t="inlineStr"/>
+      <c r="S165" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/controle</t>
+        </is>
+      </c>
+      <c r="T165" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>TIM Controle Plus 45GB</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>tim:155891</t>
+        </is>
+      </c>
+      <c r="H166" s="3" t="n">
+        <v>64.98999999999999</v>
+      </c>
+      <c r="I166" s="3" t="inlineStr"/>
+      <c r="J166" s="2" t="inlineStr"/>
+      <c r="K166" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="L166" s="2" t="inlineStr"/>
+      <c r="M166" s="2" t="inlineStr"/>
+      <c r="N166" s="2" t="inlineStr"/>
+      <c r="O166" s="2" t="inlineStr"/>
+      <c r="P166" s="2" t="inlineStr"/>
+      <c r="Q166" s="2" t="inlineStr"/>
+      <c r="R166" s="2" t="inlineStr"/>
+      <c r="S166" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/controle</t>
+        </is>
+      </c>
+      <c r="T166" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D167" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E167" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F167" s="5" t="inlineStr">
+        <is>
+          <t>TIM Controle Premium 53GB</t>
+        </is>
+      </c>
+      <c r="G167" s="5" t="inlineStr">
+        <is>
+          <t>tim:162896</t>
+        </is>
+      </c>
+      <c r="H167" s="6" t="n">
+        <v>84.98999999999999</v>
+      </c>
+      <c r="I167" s="6" t="inlineStr"/>
+      <c r="J167" s="5" t="inlineStr"/>
+      <c r="K167" s="7" t="n">
+        <v>53</v>
+      </c>
+      <c r="L167" s="5" t="inlineStr"/>
+      <c r="M167" s="5" t="inlineStr"/>
+      <c r="N167" s="5" t="inlineStr"/>
+      <c r="O167" s="5" t="inlineStr"/>
+      <c r="P167" s="5" t="inlineStr"/>
+      <c r="Q167" s="5" t="inlineStr"/>
+      <c r="R167" s="5" t="inlineStr"/>
+      <c r="S167" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/controle</t>
+        </is>
+      </c>
+      <c r="T167" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>TIM Controle Pro Express</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>tim:143576</t>
+        </is>
+      </c>
+      <c r="H168" s="3" t="n">
+        <v>64.98999999999999</v>
+      </c>
+      <c r="I168" s="3" t="inlineStr"/>
+      <c r="J168" s="2" t="inlineStr"/>
+      <c r="K168" s="4" t="inlineStr"/>
+      <c r="L168" s="2" t="inlineStr"/>
+      <c r="M168" s="2" t="inlineStr"/>
+      <c r="N168" s="2" t="inlineStr"/>
+      <c r="O168" s="2" t="inlineStr"/>
+      <c r="P168" s="2" t="inlineStr"/>
+      <c r="Q168" s="2" t="inlineStr"/>
+      <c r="R168" s="2" t="inlineStr"/>
+      <c r="S168" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/controle</t>
+        </is>
+      </c>
+      <c r="T168" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B169" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D169" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E169" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F169" s="5" t="inlineStr">
+        <is>
+          <t>TIM Black 70GB</t>
+        </is>
+      </c>
+      <c r="G169" s="5" t="inlineStr">
+        <is>
+          <t>tim:54206</t>
+        </is>
+      </c>
+      <c r="H169" s="6" t="n">
+        <v>129.99</v>
+      </c>
+      <c r="I169" s="6" t="inlineStr"/>
+      <c r="J169" s="5" t="inlineStr"/>
+      <c r="K169" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="L169" s="5" t="inlineStr"/>
+      <c r="M169" s="5" t="inlineStr"/>
+      <c r="N169" s="5" t="inlineStr"/>
+      <c r="O169" s="5" t="inlineStr"/>
+      <c r="P169" s="5" t="inlineStr"/>
+      <c r="Q169" s="5" t="inlineStr"/>
+      <c r="R169" s="5" t="inlineStr"/>
+      <c r="S169" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pos-pago/tim-black</t>
+        </is>
+      </c>
+      <c r="T169" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>TIM Black A Express 67GB</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>tim:55121</t>
+        </is>
+      </c>
+      <c r="H170" s="3" t="n">
+        <v>119.99</v>
+      </c>
+      <c r="I170" s="3" t="inlineStr"/>
+      <c r="J170" s="2" t="inlineStr"/>
+      <c r="K170" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="L170" s="2" t="inlineStr"/>
+      <c r="M170" s="2" t="inlineStr"/>
+      <c r="N170" s="2" t="inlineStr"/>
+      <c r="O170" s="2" t="inlineStr"/>
+      <c r="P170" s="2" t="inlineStr"/>
+      <c r="Q170" s="2" t="inlineStr"/>
+      <c r="R170" s="2" t="inlineStr"/>
+      <c r="S170" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pos-pago/tim-black</t>
+        </is>
+      </c>
+      <c r="T170" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B171" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C171" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D171" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F171" s="5" t="inlineStr">
+        <is>
+          <t>TIM Black B Express 82GB</t>
+        </is>
+      </c>
+      <c r="G171" s="5" t="inlineStr">
+        <is>
+          <t>tim:52146</t>
+        </is>
+      </c>
+      <c r="H171" s="6" t="n">
+        <v>144.99</v>
+      </c>
+      <c r="I171" s="6" t="inlineStr"/>
+      <c r="J171" s="5" t="inlineStr"/>
+      <c r="K171" s="7" t="n">
+        <v>82</v>
+      </c>
+      <c r="L171" s="5" t="inlineStr"/>
+      <c r="M171" s="5" t="inlineStr"/>
+      <c r="N171" s="5" t="inlineStr"/>
+      <c r="O171" s="5" t="inlineStr"/>
+      <c r="P171" s="5" t="inlineStr"/>
+      <c r="Q171" s="5" t="inlineStr"/>
+      <c r="R171" s="5" t="inlineStr"/>
+      <c r="S171" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pos-pago/tim-black</t>
+        </is>
+      </c>
+      <c r="T171" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>TIM Black C Express 107GB</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>tim:52151</t>
+        </is>
+      </c>
+      <c r="H172" s="3" t="n">
+        <v>164.99</v>
+      </c>
+      <c r="I172" s="3" t="inlineStr"/>
+      <c r="J172" s="2" t="inlineStr"/>
+      <c r="K172" s="4" t="n">
+        <v>107</v>
+      </c>
+      <c r="L172" s="2" t="inlineStr"/>
+      <c r="M172" s="2" t="inlineStr"/>
+      <c r="N172" s="2" t="inlineStr"/>
+      <c r="O172" s="2" t="inlineStr"/>
+      <c r="P172" s="2" t="inlineStr"/>
+      <c r="Q172" s="2" t="inlineStr"/>
+      <c r="R172" s="2" t="inlineStr"/>
+      <c r="S172" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pos-pago/tim-black</t>
+        </is>
+      </c>
+      <c r="T172" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B173" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C173" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D173" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E173" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F173" s="5" t="inlineStr">
+        <is>
+          <t>TIM Black C Ultra 95GB</t>
+        </is>
+      </c>
+      <c r="G173" s="5" t="inlineStr">
+        <is>
+          <t>tim:100581</t>
+        </is>
+      </c>
+      <c r="H173" s="6" t="n">
+        <v>159.99</v>
+      </c>
+      <c r="I173" s="6" t="inlineStr"/>
+      <c r="J173" s="5" t="inlineStr"/>
+      <c r="K173" s="7" t="n">
+        <v>95</v>
+      </c>
+      <c r="L173" s="5" t="inlineStr"/>
+      <c r="M173" s="5" t="inlineStr"/>
+      <c r="N173" s="5" t="inlineStr"/>
+      <c r="O173" s="5" t="inlineStr"/>
+      <c r="P173" s="5" t="inlineStr"/>
+      <c r="Q173" s="5" t="inlineStr"/>
+      <c r="R173" s="5" t="inlineStr"/>
+      <c r="S173" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pos-pago/tim-black</t>
+        </is>
+      </c>
+      <c r="T173" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>TIM Black Plus 80GB</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>tim:54256</t>
+        </is>
+      </c>
+      <c r="H174" s="3" t="n">
+        <v>149.99</v>
+      </c>
+      <c r="I174" s="3" t="inlineStr"/>
+      <c r="J174" s="2" t="inlineStr"/>
+      <c r="K174" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="L174" s="2" t="inlineStr"/>
+      <c r="M174" s="2" t="inlineStr"/>
+      <c r="N174" s="2" t="inlineStr"/>
+      <c r="O174" s="2" t="inlineStr"/>
+      <c r="P174" s="2" t="inlineStr"/>
+      <c r="Q174" s="2" t="inlineStr"/>
+      <c r="R174" s="2" t="inlineStr"/>
+      <c r="S174" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pos-pago/tim-black</t>
+        </is>
+      </c>
+      <c r="T174" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B175" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C175" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D175" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E175" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F175" s="5" t="inlineStr">
+        <is>
+          <t>TIM Black Premium 110GB</t>
+        </is>
+      </c>
+      <c r="G175" s="5" t="inlineStr">
+        <is>
+          <t>tim:54261</t>
+        </is>
+      </c>
+      <c r="H175" s="6" t="n">
+        <v>159.99</v>
+      </c>
+      <c r="I175" s="6" t="inlineStr"/>
+      <c r="J175" s="5" t="inlineStr"/>
+      <c r="K175" s="7" t="n">
+        <v>110</v>
+      </c>
+      <c r="L175" s="5" t="inlineStr"/>
+      <c r="M175" s="5" t="inlineStr"/>
+      <c r="N175" s="5" t="inlineStr"/>
+      <c r="O175" s="5" t="inlineStr"/>
+      <c r="P175" s="5" t="inlineStr"/>
+      <c r="Q175" s="5" t="inlineStr"/>
+      <c r="R175" s="5" t="inlineStr"/>
+      <c r="S175" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pos-pago/tim-black</t>
+        </is>
+      </c>
+      <c r="T175" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>TIM Pré XIP Plus 16GB</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>tim:106306</t>
+        </is>
+      </c>
+      <c r="H176" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I176" s="3" t="inlineStr"/>
+      <c r="J176" s="2" t="inlineStr"/>
+      <c r="K176" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="L176" s="2" t="inlineStr"/>
+      <c r="M176" s="2" t="inlineStr"/>
+      <c r="N176" s="2" t="inlineStr"/>
+      <c r="O176" s="2" t="inlineStr"/>
+      <c r="P176" s="2" t="inlineStr"/>
+      <c r="Q176" s="2" t="inlineStr"/>
+      <c r="R176" s="2" t="inlineStr"/>
+      <c r="S176" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pre-pago</t>
+        </is>
+      </c>
+      <c r="T176" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_prepaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B177" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C177" s="5" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D177" s="5" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E177" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F177" s="5" t="inlineStr">
+        <is>
+          <t>TIM Pré XIP Plus 6GB</t>
+        </is>
+      </c>
+      <c r="G177" s="5" t="inlineStr">
+        <is>
+          <t>tim:59906</t>
+        </is>
+      </c>
+      <c r="H177" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="I177" s="6" t="inlineStr"/>
+      <c r="J177" s="5" t="inlineStr"/>
+      <c r="K177" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="L177" s="5" t="inlineStr"/>
+      <c r="M177" s="5" t="inlineStr"/>
+      <c r="N177" s="5" t="inlineStr"/>
+      <c r="O177" s="5" t="inlineStr"/>
+      <c r="P177" s="5" t="inlineStr"/>
+      <c r="Q177" s="5" t="inlineStr"/>
+      <c r="R177" s="5" t="inlineStr"/>
+      <c r="S177" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pre-pago</t>
+        </is>
+      </c>
+      <c r="T177" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/tim_prepaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>TIM Pré XIP Plus 8GB</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>tim:59901</t>
+        </is>
+      </c>
+      <c r="H178" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="I178" s="3" t="inlineStr"/>
+      <c r="J178" s="2" t="inlineStr"/>
+      <c r="K178" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L178" s="2" t="inlineStr"/>
+      <c r="M178" s="2" t="inlineStr"/>
+      <c r="N178" s="2" t="inlineStr"/>
+      <c r="O178" s="2" t="inlineStr"/>
+      <c r="P178" s="2" t="inlineStr"/>
+      <c r="Q178" s="2" t="inlineStr"/>
+      <c r="R178" s="2" t="inlineStr"/>
+      <c r="S178" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tim.com.br/sp/para-voce/planos/pre-pago</t>
+        </is>
+      </c>
+      <c r="T178" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/tim_prepaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B179" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C179" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D179" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E179" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F179" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Controle</t>
+        </is>
+      </c>
+      <c r="G179" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029270-46gb</t>
+        </is>
+      </c>
+      <c r="H179" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="I179" s="6" t="inlineStr"/>
+      <c r="J179" s="5" t="inlineStr"/>
+      <c r="K179" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="L179" s="5" t="inlineStr">
+        <is>
+          <t>15 GB de franquia 31 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M179" s="5" t="inlineStr"/>
+      <c r="N179" s="5" t="inlineStr"/>
+      <c r="O179" s="5" t="inlineStr"/>
+      <c r="P179" s="5" t="inlineStr"/>
+      <c r="Q179" s="5" t="inlineStr"/>
+      <c r="R179" s="5" t="inlineStr">
+        <is>
+          <t>6 meses grátis de Gemini com AI Plus</t>
+        </is>
+      </c>
+      <c r="S179" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-controle</t>
+        </is>
+      </c>
+      <c r="T179" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029300-61gb</t>
+        </is>
+      </c>
+      <c r="H180" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="I180" s="3" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr"/>
+      <c r="K180" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="L180" s="2" t="inlineStr">
+        <is>
+          <t>20 GB de franquia 31 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M180" s="2" t="inlineStr"/>
+      <c r="N180" s="2" t="inlineStr"/>
+      <c r="O180" s="2" t="inlineStr"/>
+      <c r="P180" s="2" t="inlineStr"/>
+      <c r="Q180" s="2" t="inlineStr"/>
+      <c r="R180" s="2" t="inlineStr">
+        <is>
+          <t>6 meses grátis de Gemini com AI Plus</t>
+        </is>
+      </c>
+      <c r="S180" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-controle</t>
+        </is>
+      </c>
+      <c r="T180" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B181" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C181" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D181" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E181" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F181" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Controle Educação</t>
+        </is>
+      </c>
+      <c r="G181" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029273-61gb</t>
+        </is>
+      </c>
+      <c r="H181" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="I181" s="6" t="inlineStr"/>
+      <c r="J181" s="5" t="inlineStr"/>
+      <c r="K181" s="7" t="n">
+        <v>61</v>
+      </c>
+      <c r="L181" s="5" t="inlineStr">
+        <is>
+          <t>20 GB de franquia 31 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M181" s="5" t="inlineStr"/>
+      <c r="N181" s="5" t="inlineStr"/>
+      <c r="O181" s="5" t="inlineStr"/>
+      <c r="P181" s="5" t="inlineStr"/>
+      <c r="Q181" s="5" t="inlineStr"/>
+      <c r="R181" s="5" t="inlineStr">
+        <is>
+          <t>Assinatura Vivae inclusa</t>
+        </is>
+      </c>
+      <c r="S181" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-controle</t>
+        </is>
+      </c>
+      <c r="T181" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle Entretenimento</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029307-61gb</t>
+        </is>
+      </c>
+      <c r="H182" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="I182" s="3" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr"/>
+      <c r="K182" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="L182" s="2" t="inlineStr">
+        <is>
+          <t>20 GB de franquia 31 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M182" s="2" t="inlineStr"/>
+      <c r="N182" s="2" t="inlineStr"/>
+      <c r="O182" s="2" t="inlineStr"/>
+      <c r="P182" s="2" t="inlineStr"/>
+      <c r="Q182" s="2" t="inlineStr"/>
+      <c r="R182" s="2" t="inlineStr">
+        <is>
+          <t>Assinatura Vivo TV Inicial inclusa</t>
+        </is>
+      </c>
+      <c r="S182" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-controle</t>
+        </is>
+      </c>
+      <c r="T182" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B183" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C183" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D183" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E183" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F183" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Controle Música</t>
+        </is>
+      </c>
+      <c r="G183" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029313-61gb</t>
+        </is>
+      </c>
+      <c r="H183" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="I183" s="6" t="inlineStr"/>
+      <c r="J183" s="5" t="inlineStr"/>
+      <c r="K183" s="7" t="n">
+        <v>61</v>
+      </c>
+      <c r="L183" s="5" t="inlineStr">
+        <is>
+          <t>20 GB de franquia 31 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M183" s="5" t="inlineStr"/>
+      <c r="N183" s="5" t="inlineStr"/>
+      <c r="O183" s="5" t="inlineStr"/>
+      <c r="P183" s="5" t="inlineStr"/>
+      <c r="Q183" s="5" t="inlineStr"/>
+      <c r="R183" s="5" t="inlineStr">
+        <is>
+          <t>Apple Music Individual</t>
+        </is>
+      </c>
+      <c r="S183" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-controle</t>
+        </is>
+      </c>
+      <c r="T183" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle Netflix</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029308-61gb</t>
+        </is>
+      </c>
+      <c r="H184" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="I184" s="3" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr"/>
+      <c r="K184" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="L184" s="2" t="inlineStr">
+        <is>
+          <t>20 GB de franquia 31 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M184" s="2" t="inlineStr"/>
+      <c r="N184" s="2" t="inlineStr"/>
+      <c r="O184" s="2" t="inlineStr"/>
+      <c r="P184" s="2" t="inlineStr"/>
+      <c r="Q184" s="2" t="inlineStr"/>
+      <c r="R184" s="2" t="inlineStr">
+        <is>
+          <t>Assinatura Netflix Padrão com anúncios</t>
+        </is>
+      </c>
+      <c r="S184" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-controle</t>
+        </is>
+      </c>
+      <c r="T184" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B185" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C185" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D185" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F185" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Controle Saúde</t>
+        </is>
+      </c>
+      <c r="G185" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029301-61gb</t>
+        </is>
+      </c>
+      <c r="H185" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="I185" s="6" t="inlineStr"/>
+      <c r="J185" s="5" t="inlineStr"/>
+      <c r="K185" s="7" t="n">
+        <v>61</v>
+      </c>
+      <c r="L185" s="5" t="inlineStr">
+        <is>
+          <t>20 GB de franquia 31 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M185" s="5" t="inlineStr"/>
+      <c r="N185" s="5" t="inlineStr"/>
+      <c r="O185" s="5" t="inlineStr"/>
+      <c r="P185" s="5" t="inlineStr"/>
+      <c r="Q185" s="5" t="inlineStr"/>
+      <c r="R185" s="5" t="inlineStr">
+        <is>
+          <t>Assinatura Vale Saúde Sempre inclusa</t>
+        </is>
+      </c>
+      <c r="S185" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-controle</t>
+        </is>
+      </c>
+      <c r="T185" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_control_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>lite</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>Easy Lite</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600025883-30gb</t>
+        </is>
+      </c>
+      <c r="H186" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I186" s="3" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr"/>
+      <c r="K186" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="L186" s="2" t="inlineStr">
+        <is>
+          <t>30 GB de franquia</t>
+        </is>
+      </c>
+      <c r="M186" s="2" t="inlineStr"/>
+      <c r="N186" s="2" t="inlineStr"/>
+      <c r="O186" s="2" t="inlineStr"/>
+      <c r="P186" s="2" t="inlineStr"/>
+      <c r="Q186" s="2" t="inlineStr"/>
+      <c r="R186" s="2" t="inlineStr">
+        <is>
+          <t>2 meses de YouTube sem consumo no plano</t>
+        </is>
+      </c>
+      <c r="S186" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/easy-lite</t>
+        </is>
+      </c>
+      <c r="T186" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_lite_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B187" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C187" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D187" s="5" t="inlineStr">
+        <is>
+          <t>lite</t>
+        </is>
+      </c>
+      <c r="E187" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F187" s="5" t="inlineStr">
+        <is>
+          <t>Easy Lite</t>
+        </is>
+      </c>
+      <c r="G187" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600025885-40gb</t>
+        </is>
+      </c>
+      <c r="H187" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="I187" s="6" t="inlineStr"/>
+      <c r="J187" s="5" t="inlineStr"/>
+      <c r="K187" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="L187" s="5" t="inlineStr">
+        <is>
+          <t>40 GB de franquia</t>
+        </is>
+      </c>
+      <c r="M187" s="5" t="inlineStr"/>
+      <c r="N187" s="5" t="inlineStr"/>
+      <c r="O187" s="5" t="inlineStr"/>
+      <c r="P187" s="5" t="inlineStr"/>
+      <c r="Q187" s="5" t="inlineStr"/>
+      <c r="R187" s="5" t="inlineStr">
+        <is>
+          <t>2 meses de YouTube sem consumo no plano</t>
+        </is>
+      </c>
+      <c r="S187" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/easy-lite</t>
+        </is>
+      </c>
+      <c r="T187" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_lite_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>lite</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>Easy Lite</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600025888-20gb</t>
+        </is>
+      </c>
+      <c r="H188" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="I188" s="3" t="inlineStr"/>
+      <c r="J188" s="2" t="inlineStr"/>
+      <c r="K188" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="L188" s="2" t="inlineStr">
+        <is>
+          <t>20 GB de franquia</t>
+        </is>
+      </c>
+      <c r="M188" s="2" t="inlineStr"/>
+      <c r="N188" s="2" t="inlineStr"/>
+      <c r="O188" s="2" t="inlineStr"/>
+      <c r="P188" s="2" t="inlineStr"/>
+      <c r="Q188" s="2" t="inlineStr"/>
+      <c r="R188" s="2" t="inlineStr">
+        <is>
+          <t>2 meses de YouTube sem consumo no plano</t>
+        </is>
+      </c>
+      <c r="S188" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/easy-lite</t>
+        </is>
+      </c>
+      <c r="T188" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_lite_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B189" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C189" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D189" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E189" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F189" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Pós com Amazon</t>
+        </is>
+      </c>
+      <c r="G189" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029255-60gb</t>
+        </is>
+      </c>
+      <c r="H189" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I189" s="6" t="inlineStr"/>
+      <c r="J189" s="5" t="inlineStr"/>
+      <c r="K189" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="L189" s="5" t="inlineStr">
+        <is>
+          <t>50 GB de franquia 10 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M189" s="5" t="inlineStr"/>
+      <c r="N189" s="5" t="inlineStr"/>
+      <c r="O189" s="5" t="inlineStr"/>
+      <c r="P189" s="5" t="inlineStr"/>
+      <c r="Q189" s="5" t="inlineStr"/>
+      <c r="R189" s="5" t="inlineStr">
+        <is>
+          <t>Assinatura Amazon Prime inclusa</t>
+        </is>
+      </c>
+      <c r="S189" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-pos-pago</t>
+        </is>
+      </c>
+      <c r="T189" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Pós com Disney+</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600022115-60gb</t>
+        </is>
+      </c>
+      <c r="H190" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="I190" s="3" t="inlineStr"/>
+      <c r="J190" s="2" t="inlineStr"/>
+      <c r="K190" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="L190" s="2" t="inlineStr">
+        <is>
+          <t>50 GB de franquia 10 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M190" s="2" t="inlineStr"/>
+      <c r="N190" s="2" t="inlineStr"/>
+      <c r="O190" s="2" t="inlineStr"/>
+      <c r="P190" s="2" t="inlineStr">
+        <is>
+          <t>Disney+</t>
+        </is>
+      </c>
+      <c r="Q190" s="2" t="inlineStr"/>
+      <c r="R190" s="2" t="inlineStr">
+        <is>
+          <t>Assinatura Disney+ Padrão inclusa</t>
+        </is>
+      </c>
+      <c r="S190" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-pos-pago</t>
+        </is>
+      </c>
+      <c r="T190" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D191" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E191" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F191" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Pós com Globoplay</t>
+        </is>
+      </c>
+      <c r="G191" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029246-60gb</t>
+        </is>
+      </c>
+      <c r="H191" s="6" t="n">
+        <v>165</v>
+      </c>
+      <c r="I191" s="6" t="inlineStr"/>
+      <c r="J191" s="5" t="inlineStr"/>
+      <c r="K191" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="L191" s="5" t="inlineStr">
+        <is>
+          <t>50 GB de franquia 10 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M191" s="5" t="inlineStr"/>
+      <c r="N191" s="5" t="inlineStr"/>
+      <c r="O191" s="5" t="inlineStr"/>
+      <c r="P191" s="5" t="inlineStr">
+        <is>
+          <t>Globoplay</t>
+        </is>
+      </c>
+      <c r="Q191" s="5" t="inlineStr"/>
+      <c r="R191" s="5" t="inlineStr">
+        <is>
+          <t>Assinatura Globoplay inclusa</t>
+        </is>
+      </c>
+      <c r="S191" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-pos-pago</t>
+        </is>
+      </c>
+      <c r="T191" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Pós com Netflix</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029234-60gb</t>
+        </is>
+      </c>
+      <c r="H192" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="I192" s="3" t="inlineStr"/>
+      <c r="J192" s="2" t="inlineStr"/>
+      <c r="K192" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="L192" s="2" t="inlineStr">
+        <is>
+          <t>50 GB de franquia 10 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M192" s="2" t="inlineStr"/>
+      <c r="N192" s="2" t="inlineStr"/>
+      <c r="O192" s="2" t="inlineStr"/>
+      <c r="P192" s="2" t="inlineStr">
+        <is>
+          <t>Netflix</t>
+        </is>
+      </c>
+      <c r="Q192" s="2" t="inlineStr"/>
+      <c r="R192" s="2" t="inlineStr">
+        <is>
+          <t>Assinatura Netflix Padrão inclusa</t>
+        </is>
+      </c>
+      <c r="S192" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-pos-pago</t>
+        </is>
+      </c>
+      <c r="T192" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D193" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F193" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Pós com Premiere</t>
+        </is>
+      </c>
+      <c r="G193" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029249-60gb</t>
+        </is>
+      </c>
+      <c r="H193" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="I193" s="6" t="inlineStr"/>
+      <c r="J193" s="5" t="inlineStr"/>
+      <c r="K193" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="L193" s="5" t="inlineStr">
+        <is>
+          <t>50 GB de franquia 10 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M193" s="5" t="inlineStr"/>
+      <c r="N193" s="5" t="inlineStr"/>
+      <c r="O193" s="5" t="inlineStr"/>
+      <c r="P193" s="5" t="inlineStr">
+        <is>
+          <t>Premiere</t>
+        </is>
+      </c>
+      <c r="Q193" s="5" t="inlineStr"/>
+      <c r="R193" s="5" t="inlineStr">
+        <is>
+          <t>Assinatura Premiere inclusa</t>
+        </is>
+      </c>
+      <c r="S193" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-pos-pago</t>
+        </is>
+      </c>
+      <c r="T193" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Pós com Spotify</t>
+        </is>
+      </c>
+      <c r="G194" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029229-60gb</t>
+        </is>
+      </c>
+      <c r="H194" s="3" t="n">
+        <v>165</v>
+      </c>
+      <c r="I194" s="3" t="inlineStr"/>
+      <c r="J194" s="2" t="inlineStr"/>
+      <c r="K194" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="L194" s="2" t="inlineStr">
+        <is>
+          <t>50 GB de franquia 10 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M194" s="2" t="inlineStr"/>
+      <c r="N194" s="2" t="inlineStr"/>
+      <c r="O194" s="2" t="inlineStr"/>
+      <c r="P194" s="2" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="Q194" s="2" t="inlineStr"/>
+      <c r="R194" s="2" t="inlineStr">
+        <is>
+          <t>Assinatura Spotify Premium inclusa</t>
+        </is>
+      </c>
+      <c r="S194" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-pos-pago</t>
+        </is>
+      </c>
+      <c r="T194" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B195" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C195" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D195" s="5" t="inlineStr">
+        <is>
+          <t>postpaid</t>
+        </is>
+      </c>
+      <c r="E195" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F195" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Pós com Travel</t>
+        </is>
+      </c>
+      <c r="G195" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029244-70gb</t>
+        </is>
+      </c>
+      <c r="H195" s="6" t="n">
+        <v>215</v>
+      </c>
+      <c r="I195" s="6" t="inlineStr"/>
+      <c r="J195" s="5" t="inlineStr"/>
+      <c r="K195" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="L195" s="5" t="inlineStr">
+        <is>
+          <t>60 GB de franquia 10 GB de bônus</t>
+        </is>
+      </c>
+      <c r="M195" s="5" t="inlineStr"/>
+      <c r="N195" s="5" t="inlineStr"/>
+      <c r="O195" s="5" t="inlineStr"/>
+      <c r="P195" s="5" t="inlineStr"/>
+      <c r="Q195" s="5" t="inlineStr"/>
+      <c r="R195" s="5" t="inlineStr">
+        <is>
+          <t>6 meses grátis de Gemini com AI Plus</t>
+        </is>
+      </c>
+      <c r="S195" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/planos-pos-pago</t>
+        </is>
+      </c>
+      <c r="T195" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_postpaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Pré</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029370-25gb</t>
+        </is>
+      </c>
+      <c r="H196" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I196" s="3" t="inlineStr"/>
+      <c r="J196" s="2" t="inlineStr"/>
+      <c r="K196" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="L196" s="2" t="inlineStr">
+        <is>
+          <t>15 GB para navegar como quiser 5 GB de bônus 5 GB para navegar no Youtube</t>
+        </is>
+      </c>
+      <c r="M196" s="2" t="inlineStr"/>
+      <c r="N196" s="2" t="inlineStr"/>
+      <c r="O196" s="2" t="inlineStr"/>
+      <c r="P196" s="2" t="inlineStr"/>
+      <c r="Q196" s="2" t="inlineStr"/>
+      <c r="R196" s="2" t="inlineStr"/>
+      <c r="S196" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/pre-pago/vivo-pre</t>
+        </is>
+      </c>
+      <c r="T196" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_prepaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B197" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C197" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D197" s="5" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E197" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F197" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Pré</t>
+        </is>
+      </c>
+      <c r="G197" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029370-9gb</t>
+        </is>
+      </c>
+      <c r="H197" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="I197" s="6" t="inlineStr"/>
+      <c r="J197" s="5" t="inlineStr"/>
+      <c r="K197" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="L197" s="5" t="inlineStr">
+        <is>
+          <t>6 GB para navegar como quiser 3 GB para navegar no YouTube</t>
+        </is>
+      </c>
+      <c r="M197" s="5" t="inlineStr"/>
+      <c r="N197" s="5" t="inlineStr"/>
+      <c r="O197" s="5" t="inlineStr"/>
+      <c r="P197" s="5" t="inlineStr"/>
+      <c r="Q197" s="5" t="inlineStr"/>
+      <c r="R197" s="5" t="inlineStr"/>
+      <c r="S197" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/pre-pago/vivo-pre</t>
+        </is>
+      </c>
+      <c r="T197" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_prepaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Pré</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029370-5gb</t>
+        </is>
+      </c>
+      <c r="H198" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I198" s="3" t="inlineStr"/>
+      <c r="J198" s="2" t="inlineStr"/>
+      <c r="K198" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L198" s="2" t="inlineStr">
+        <is>
+          <t>5 GB para navegar como quiser</t>
+        </is>
+      </c>
+      <c r="M198" s="2" t="inlineStr"/>
+      <c r="N198" s="2" t="inlineStr"/>
+      <c r="O198" s="2" t="inlineStr"/>
+      <c r="P198" s="2" t="inlineStr"/>
+      <c r="Q198" s="2" t="inlineStr"/>
+      <c r="R198" s="2" t="inlineStr"/>
+      <c r="S198" s="2" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/pre-pago/vivo-pre</t>
+        </is>
+      </c>
+      <c r="T198" s="2" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_prepaid_SP.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B199" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:19:40</t>
+        </is>
+      </c>
+      <c r="C199" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="D199" s="5" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="E199" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F199" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Pré</t>
+        </is>
+      </c>
+      <c r="G199" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029370-4gb</t>
+        </is>
+      </c>
+      <c r="H199" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="I199" s="6" t="inlineStr"/>
+      <c r="J199" s="5" t="inlineStr"/>
+      <c r="K199" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L199" s="5" t="inlineStr">
+        <is>
+          <t>4 GB para navegar como quiser</t>
+        </is>
+      </c>
+      <c r="M199" s="5" t="inlineStr"/>
+      <c r="N199" s="5" t="inlineStr"/>
+      <c r="O199" s="5" t="inlineStr"/>
+      <c r="P199" s="5" t="inlineStr"/>
+      <c r="Q199" s="5" t="inlineStr"/>
+      <c r="R199" s="5" t="inlineStr"/>
+      <c r="S199" s="5" t="inlineStr">
+        <is>
+          <t>https://vivo.com.br/para-voce/produtos-e-servicos/para-o-celular/pre-pago/vivo-pre</t>
+        </is>
+      </c>
+      <c r="T199" s="5" t="inlineStr">
+        <is>
+          <t>data/raw/vivo_prepaid_SP.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T150"/>
+  <autoFilter ref="A1:T199"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11743,12 +15057,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -11819,12 +15133,12 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -11889,12 +15203,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -11959,12 +15273,12 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -12029,12 +15343,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -12099,12 +15413,12 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -12169,12 +15483,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -12239,12 +15553,12 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -12309,12 +15623,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -12379,12 +15693,12 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -12449,12 +15763,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -12519,12 +15833,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -12589,12 +15903,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -12655,12 +15969,12 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -12717,12 +16031,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -12779,12 +16093,12 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -12841,12 +16155,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -12903,12 +16217,12 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -12963,12 +16277,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -13025,12 +16339,12 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -13087,12 +16401,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -13149,12 +16463,12 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -13211,12 +16525,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -13273,12 +16587,12 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -13335,12 +16649,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -13397,12 +16711,12 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -13459,12 +16773,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -13521,12 +16835,12 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -13583,12 +16897,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -13653,12 +16967,12 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -13723,12 +17037,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -13793,12 +17107,12 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -13863,12 +17177,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -13933,12 +17247,12 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -14003,12 +17317,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -14073,12 +17387,12 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -14126,7 +17440,7 @@
       <c r="Q37" s="5" t="inlineStr"/>
       <c r="R37" s="5" t="inlineStr">
         <is>
-          <t>2 meses de YouTube sem desconto no plano</t>
+          <t>2 meses de YouTube sem consumo no plano</t>
         </is>
       </c>
       <c r="S37" s="5" t="inlineStr">
@@ -14143,12 +17457,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -14196,7 +17510,7 @@
       <c r="Q38" s="2" t="inlineStr"/>
       <c r="R38" s="2" t="inlineStr">
         <is>
-          <t>2 meses de YouTube sem desconto no plano</t>
+          <t>2 meses de YouTube sem consumo no plano</t>
         </is>
       </c>
       <c r="S38" s="2" t="inlineStr">
@@ -14213,12 +17527,12 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -14266,7 +17580,7 @@
       <c r="Q39" s="5" t="inlineStr"/>
       <c r="R39" s="5" t="inlineStr">
         <is>
-          <t>2 meses de YouTube sem desconto no plano</t>
+          <t>2 meses de YouTube sem consumo no plano</t>
         </is>
       </c>
       <c r="S39" s="5" t="inlineStr">
@@ -14283,12 +17597,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -14353,12 +17667,12 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -14427,12 +17741,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -14501,12 +17815,12 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -14575,12 +17889,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -14649,12 +17963,12 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -14723,12 +18037,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -14793,12 +18107,12 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -14823,7 +18137,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600022379-25gb</t>
+          <t>vivo:VIV202600029370-25gb</t>
         </is>
       </c>
       <c r="H47" s="6" t="n">
@@ -14859,12 +18173,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -14889,7 +18203,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600022379-9gb</t>
+          <t>vivo:VIV202600029370-9gb</t>
         </is>
       </c>
       <c r="H48" s="3" t="n">
@@ -14925,12 +18239,12 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -14955,7 +18269,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600022379-5gb</t>
+          <t>vivo:VIV202600029370-5gb</t>
         </is>
       </c>
       <c r="H49" s="6" t="n">
@@ -14991,12 +18305,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -15021,7 +18335,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600022379-4gb</t>
+          <t>vivo:VIV202600029370-4gb</t>
         </is>
       </c>
       <c r="H50" s="3" t="n">
@@ -15084,7 +18398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15158,7 +18472,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>lite</t>
+          <t>prepaid</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -15168,12 +18482,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600025883-30gb</t>
+          <t>vivo:VIV202600029370-25gb</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Easy Lite</t>
+          <t>Vivo Pré</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr"/>
@@ -15195,7 +18509,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>lite</t>
+          <t>prepaid</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -15205,17 +18519,17 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600025885-40gb</t>
+          <t>vivo:VIV202600029370-4gb</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Easy Lite</t>
+          <t>Vivo Pré</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr"/>
       <c r="H3" s="6" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="I3" s="6" t="inlineStr"/>
     </row>
@@ -15232,7 +18546,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>lite</t>
+          <t>prepaid</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -15242,24 +18556,24 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600025888-20gb</t>
+          <t>vivo:VIV202600029370-5gb</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Easy Lite</t>
+          <t>Vivo Pré</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="3" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="I4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>removed</t>
+          <t>new</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -15269,7 +18583,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>lite</t>
+          <t>prepaid</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -15279,18 +18593,18 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600005312-30gb</t>
+          <t>vivo:VIV202600029370-9gb</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Easy Lite</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="H5" s="6" t="inlineStr"/>
+          <t>Vivo Pré</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="n">
+        <v>25</v>
+      </c>
       <c r="I5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
@@ -15306,7 +18620,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>lite</t>
+          <t>prepaid</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -15316,16 +18630,16 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600019132-20gb</t>
+          <t>vivo:VIV202600022379-25gb</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Easy Lite</t>
+          <t>Vivo Pré</t>
         </is>
       </c>
       <c r="G6" s="3" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr"/>
@@ -15343,7 +18657,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>lite</t>
+          <t>prepaid</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -15353,19 +18667,93 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600019134-40gb</t>
+          <t>vivo:VIV202600022379-4gb</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Easy Lite</t>
+          <t>Vivo Pré</t>
         </is>
       </c>
       <c r="G7" s="6" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600022379-5gb</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Pré</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>prepaid</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600022379-9gb</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Pré</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15404,7 +18792,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T22:14:36</t>
+          <t>2026-06-25T22:19:40</t>
         </is>
       </c>
     </row>
@@ -15416,7 +18804,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -15437,7 +18825,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -15548,7 +18936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15836,8 +19224,63 @@
         <v/>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="12" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B40" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"control",history!$A:$A,$A40)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"control",history!$A:$A,$A40))</f>
+        <v/>
+      </c>
+      <c r="C40" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"control",history!$A:$A,$A40)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"control",history!$A:$A,$A40))</f>
+        <v/>
+      </c>
+      <c r="D40" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"control",history!$A:$A,$A40)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"control",history!$A:$A,$A40))</f>
+        <v/>
+      </c>
+      <c r="E40" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"postpaid",history!$A:$A,$A40)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"postpaid",history!$A:$A,$A40))</f>
+        <v/>
+      </c>
+      <c r="F40" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"postpaid",history!$A:$A,$A40)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"postpaid",history!$A:$A,$A40))</f>
+        <v/>
+      </c>
+      <c r="G40" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"postpaid",history!$A:$A,$A40)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"postpaid",history!$A:$A,$A40))</f>
+        <v/>
+      </c>
+      <c r="H40" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"prepaid",history!$A:$A,$A40)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"prepaid",history!$A:$A,$A40))</f>
+        <v/>
+      </c>
+      <c r="I40" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"prepaid",history!$A:$A,$A40)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"prepaid",history!$A:$A,$A40))</f>
+        <v/>
+      </c>
+      <c r="J40" s="3">
+        <f>IF(_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"prepaid",history!$A:$A,$A40)=0,"",_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"prepaid",history!$A:$A,$A40))</f>
+        <v/>
+      </c>
+      <c r="K40" s="3">
+        <f>IFERROR(1/MAX(IFERROR(1/_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"lite",history!$A:$A,$A40),0),IFERROR(1/_xlfn.MINIFS(history!$H:$H,history!$C:$C,"tim",history!$D:$D,"flex",history!$A:$A,$A40),0)),"")</f>
+        <v/>
+      </c>
+      <c r="L40" s="3">
+        <f>IFERROR(1/MAX(IFERROR(1/_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"lite",history!$A:$A,$A40),0),IFERROR(1/_xlfn.MINIFS(history!$H:$H,history!$C:$C,"vivo",history!$D:$D,"flex",history!$A:$A,$A40),0)),"")</f>
+        <v/>
+      </c>
+      <c r="M40" s="3">
+        <f>IFERROR(1/MAX(IFERROR(1/_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"lite",history!$A:$A,$A40),0),IFERROR(1/_xlfn.MINIFS(history!$H:$H,history!$C:$C,"claro",history!$D:$D,"flex",history!$A:$A,$A40),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
         <is>
           <t>Pre = cheapest recharge amount captured (true R$/day needs validity-days we don't yet capture — CONTEXT §8). Digital = min of Vivo Lite / Claro Flex. Daily rows now; monthly roll-up is the planned next step.</t>
         </is>
@@ -15851,7 +19294,7 @@
     <mergeCell ref="K35:M35"/>
     <mergeCell ref="H35:J35"/>
   </mergeCells>
-  <conditionalFormatting sqref="B37:D39">
+  <conditionalFormatting sqref="B37:D40">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -15863,7 +19306,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E37:G39">
+  <conditionalFormatting sqref="E37:G40">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -15875,7 +19318,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H37:J39">
+  <conditionalFormatting sqref="H37:J40">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -15887,7 +19330,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K37:M39">
+  <conditionalFormatting sqref="K37:M40">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -17187,7 +20630,7 @@
       <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2 meses de YouTube sem desconto no plano</t>
+          <t>2 meses de YouTube sem consumo no plano</t>
         </is>
       </c>
     </row>
@@ -17211,7 +20654,7 @@
       <c r="G20" s="5" t="n"/>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>2 meses de YouTube sem desconto no plano</t>
+          <t>2 meses de YouTube sem consumo no plano</t>
         </is>
       </c>
     </row>
@@ -17235,7 +20678,7 @@
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2 meses de YouTube sem desconto no plano</t>
+          <t>2 meses de YouTube sem consumo no plano</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): daily snapshot 2026-07-01
</commit_message>
<xml_diff>
--- a/projects/mobile-price-tracker/data/mobile_plans.xlsx
+++ b/projects/mobile-price-tracker/data/mobile_plans.xlsx
@@ -34753,7 +34753,7 @@
       </c>
       <c r="B475" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C475" s="5" t="inlineStr">
@@ -34831,7 +34831,7 @@
       </c>
       <c r="B476" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C476" s="2" t="inlineStr">
@@ -34903,7 +34903,7 @@
       </c>
       <c r="B477" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C477" s="5" t="inlineStr">
@@ -34975,7 +34975,7 @@
       </c>
       <c r="B478" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C478" s="2" t="inlineStr">
@@ -35047,7 +35047,7 @@
       </c>
       <c r="B479" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C479" s="5" t="inlineStr">
@@ -35119,7 +35119,7 @@
       </c>
       <c r="B480" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C480" s="2" t="inlineStr">
@@ -35191,7 +35191,7 @@
       </c>
       <c r="B481" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C481" s="5" t="inlineStr">
@@ -35263,7 +35263,7 @@
       </c>
       <c r="B482" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C482" s="2" t="inlineStr">
@@ -35335,7 +35335,7 @@
       </c>
       <c r="B483" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C483" s="5" t="inlineStr">
@@ -35407,7 +35407,7 @@
       </c>
       <c r="B484" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C484" s="2" t="inlineStr">
@@ -35479,7 +35479,7 @@
       </c>
       <c r="B485" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C485" s="5" t="inlineStr">
@@ -35551,7 +35551,7 @@
       </c>
       <c r="B486" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C486" s="2" t="inlineStr">
@@ -35623,7 +35623,7 @@
       </c>
       <c r="B487" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C487" s="5" t="inlineStr">
@@ -35693,7 +35693,7 @@
       </c>
       <c r="B488" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C488" s="2" t="inlineStr">
@@ -35763,7 +35763,7 @@
       </c>
       <c r="B489" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C489" s="5" t="inlineStr">
@@ -35833,7 +35833,7 @@
       </c>
       <c r="B490" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C490" s="2" t="inlineStr">
@@ -35903,7 +35903,7 @@
       </c>
       <c r="B491" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C491" s="5" t="inlineStr">
@@ -35973,7 +35973,7 @@
       </c>
       <c r="B492" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C492" s="2" t="inlineStr">
@@ -36043,7 +36043,7 @@
       </c>
       <c r="B493" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C493" s="5" t="inlineStr">
@@ -36113,7 +36113,7 @@
       </c>
       <c r="B494" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C494" s="2" t="inlineStr">
@@ -36177,7 +36177,7 @@
       </c>
       <c r="B495" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C495" s="5" t="inlineStr">
@@ -36241,7 +36241,7 @@
       </c>
       <c r="B496" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C496" s="2" t="inlineStr">
@@ -36305,7 +36305,7 @@
       </c>
       <c r="B497" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C497" s="5" t="inlineStr">
@@ -36369,7 +36369,7 @@
       </c>
       <c r="B498" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C498" s="2" t="inlineStr">
@@ -36431,7 +36431,7 @@
       </c>
       <c r="B499" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C499" s="5" t="inlineStr">
@@ -36499,7 +36499,7 @@
       </c>
       <c r="B500" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C500" s="2" t="inlineStr">
@@ -36567,7 +36567,7 @@
       </c>
       <c r="B501" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C501" s="5" t="inlineStr">
@@ -36635,7 +36635,7 @@
       </c>
       <c r="B502" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C502" s="2" t="inlineStr">
@@ -36703,7 +36703,7 @@
       </c>
       <c r="B503" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C503" s="5" t="inlineStr">
@@ -36771,7 +36771,7 @@
       </c>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C504" s="2" t="inlineStr">
@@ -36839,7 +36839,7 @@
       </c>
       <c r="B505" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C505" s="5" t="inlineStr">
@@ -36907,7 +36907,7 @@
       </c>
       <c r="B506" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C506" s="2" t="inlineStr">
@@ -36973,7 +36973,7 @@
       </c>
       <c r="B507" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C507" s="5" t="inlineStr">
@@ -37039,7 +37039,7 @@
       </c>
       <c r="B508" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C508" s="2" t="inlineStr">
@@ -37105,7 +37105,7 @@
       </c>
       <c r="B509" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C509" s="5" t="inlineStr">
@@ -37177,7 +37177,7 @@
       </c>
       <c r="B510" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C510" s="2" t="inlineStr">
@@ -37202,17 +37202,17 @@
       </c>
       <c r="G510" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029300-51gb</t>
+          <t>vivo:VIV202600029300-61gb</t>
         </is>
       </c>
       <c r="H510" s="3" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="I510" s="3" t="inlineStr"/>
       <c r="J510" s="2" t="inlineStr"/>
       <c r="K510" s="2" t="inlineStr"/>
       <c r="L510" s="4" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M510" s="2" t="inlineStr">
         <is>
@@ -37249,7 +37249,7 @@
       </c>
       <c r="B511" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C511" s="5" t="inlineStr">
@@ -37274,17 +37274,17 @@
       </c>
       <c r="G511" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029273-51gb</t>
+          <t>vivo:VIV202600029273-61gb</t>
         </is>
       </c>
       <c r="H511" s="6" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="I511" s="6" t="inlineStr"/>
       <c r="J511" s="5" t="inlineStr"/>
       <c r="K511" s="5" t="inlineStr"/>
       <c r="L511" s="7" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M511" s="5" t="inlineStr">
         <is>
@@ -37321,7 +37321,7 @@
       </c>
       <c r="B512" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C512" s="2" t="inlineStr">
@@ -37346,17 +37346,17 @@
       </c>
       <c r="G512" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029307-51gb</t>
+          <t>vivo:VIV202600029307-61gb</t>
         </is>
       </c>
       <c r="H512" s="3" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="I512" s="3" t="inlineStr"/>
       <c r="J512" s="2" t="inlineStr"/>
       <c r="K512" s="2" t="inlineStr"/>
       <c r="L512" s="4" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M512" s="2" t="inlineStr">
         <is>
@@ -37393,7 +37393,7 @@
       </c>
       <c r="B513" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C513" s="5" t="inlineStr">
@@ -37418,17 +37418,17 @@
       </c>
       <c r="G513" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029313-51gb</t>
+          <t>vivo:VIV202600029313-61gb</t>
         </is>
       </c>
       <c r="H513" s="6" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="I513" s="6" t="inlineStr"/>
       <c r="J513" s="5" t="inlineStr"/>
       <c r="K513" s="5" t="inlineStr"/>
       <c r="L513" s="7" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M513" s="5" t="inlineStr">
         <is>
@@ -37465,7 +37465,7 @@
       </c>
       <c r="B514" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C514" s="2" t="inlineStr">
@@ -37490,17 +37490,17 @@
       </c>
       <c r="G514" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029308-51gb</t>
+          <t>vivo:VIV202600029308-61gb</t>
         </is>
       </c>
       <c r="H514" s="3" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="I514" s="3" t="inlineStr"/>
       <c r="J514" s="2" t="inlineStr"/>
       <c r="K514" s="2" t="inlineStr"/>
       <c r="L514" s="4" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M514" s="2" t="inlineStr">
         <is>
@@ -37537,7 +37537,7 @@
       </c>
       <c r="B515" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C515" s="5" t="inlineStr">
@@ -37562,17 +37562,17 @@
       </c>
       <c r="G515" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029301-51gb</t>
+          <t>vivo:VIV202600029301-61gb</t>
         </is>
       </c>
       <c r="H515" s="6" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="I515" s="6" t="inlineStr"/>
       <c r="J515" s="5" t="inlineStr"/>
       <c r="K515" s="5" t="inlineStr"/>
       <c r="L515" s="7" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M515" s="5" t="inlineStr">
         <is>
@@ -37609,7 +37609,7 @@
       </c>
       <c r="B516" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C516" s="2" t="inlineStr">
@@ -37634,17 +37634,17 @@
       </c>
       <c r="G516" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029274-51gb</t>
+          <t>vivo:VIV202600029274-61gb</t>
         </is>
       </c>
       <c r="H516" s="3" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="I516" s="3" t="inlineStr"/>
       <c r="J516" s="2" t="inlineStr"/>
       <c r="K516" s="2" t="inlineStr"/>
       <c r="L516" s="4" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M516" s="2" t="inlineStr">
         <is>
@@ -37681,7 +37681,7 @@
       </c>
       <c r="B517" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C517" s="5" t="inlineStr">
@@ -37706,7 +37706,7 @@
       </c>
       <c r="G517" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600025883-30gb</t>
+          <t>vivo:VIV202600032594-30gb</t>
         </is>
       </c>
       <c r="H517" s="6" t="n">
@@ -37761,7 +37761,7 @@
       </c>
       <c r="B518" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C518" s="2" t="inlineStr">
@@ -37786,7 +37786,7 @@
       </c>
       <c r="G518" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600025885-40gb</t>
+          <t>vivo:VIV202600032596-40gb</t>
         </is>
       </c>
       <c r="H518" s="3" t="n">
@@ -37841,7 +37841,7 @@
       </c>
       <c r="B519" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C519" s="5" t="inlineStr">
@@ -37866,7 +37866,7 @@
       </c>
       <c r="G519" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600025888-20gb</t>
+          <t>vivo:VIV202600032599-20gb</t>
         </is>
       </c>
       <c r="H519" s="6" t="n">
@@ -37913,7 +37913,7 @@
       </c>
       <c r="B520" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C520" s="2" t="inlineStr">
@@ -37985,7 +37985,7 @@
       </c>
       <c r="B521" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C521" s="5" t="inlineStr">
@@ -38061,7 +38061,7 @@
       </c>
       <c r="B522" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C522" s="2" t="inlineStr">
@@ -38137,7 +38137,7 @@
       </c>
       <c r="B523" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C523" s="5" t="inlineStr">
@@ -38213,7 +38213,7 @@
       </c>
       <c r="B524" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C524" s="2" t="inlineStr">
@@ -38289,7 +38289,7 @@
       </c>
       <c r="B525" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C525" s="5" t="inlineStr">
@@ -38365,7 +38365,7 @@
       </c>
       <c r="B526" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C526" s="2" t="inlineStr">
@@ -38437,7 +38437,7 @@
       </c>
       <c r="B527" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C527" s="5" t="inlineStr">
@@ -38507,7 +38507,7 @@
       </c>
       <c r="B528" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C528" s="2" t="inlineStr">
@@ -38577,7 +38577,7 @@
       </c>
       <c r="B529" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C529" s="5" t="inlineStr">
@@ -38647,7 +38647,7 @@
       </c>
       <c r="B530" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C530" s="2" t="inlineStr">
@@ -39310,7 +39310,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -39388,7 +39388,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -39460,7 +39460,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -39532,7 +39532,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -39604,7 +39604,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -39676,7 +39676,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -39748,7 +39748,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -39820,7 +39820,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -39892,7 +39892,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -39964,7 +39964,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -40036,7 +40036,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -40108,7 +40108,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -40180,7 +40180,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -40250,7 +40250,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -40320,7 +40320,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -40390,7 +40390,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -40460,7 +40460,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -40530,7 +40530,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -40600,7 +40600,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -40670,7 +40670,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -40734,7 +40734,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -40798,7 +40798,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -40862,7 +40862,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -40926,7 +40926,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -40988,7 +40988,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -41056,7 +41056,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -41124,7 +41124,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -41192,7 +41192,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -41260,7 +41260,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -41328,7 +41328,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -41396,7 +41396,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -41464,7 +41464,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -41530,7 +41530,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -41596,7 +41596,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -41662,7 +41662,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -41734,7 +41734,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -41759,17 +41759,17 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029300-51gb</t>
+          <t>vivo:VIV202600029300-61gb</t>
         </is>
       </c>
       <c r="H37" s="6" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="I37" s="6" t="inlineStr"/>
       <c r="J37" s="5" t="inlineStr"/>
       <c r="K37" s="5" t="inlineStr"/>
       <c r="L37" s="7" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M37" s="5" t="inlineStr">
         <is>
@@ -41806,7 +41806,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -41831,17 +41831,17 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029273-51gb</t>
+          <t>vivo:VIV202600029273-61gb</t>
         </is>
       </c>
       <c r="H38" s="3" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="I38" s="3" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="4" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
@@ -41878,7 +41878,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -41903,17 +41903,17 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029307-51gb</t>
+          <t>vivo:VIV202600029307-61gb</t>
         </is>
       </c>
       <c r="H39" s="6" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="I39" s="6" t="inlineStr"/>
       <c r="J39" s="5" t="inlineStr"/>
       <c r="K39" s="5" t="inlineStr"/>
       <c r="L39" s="7" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M39" s="5" t="inlineStr">
         <is>
@@ -41950,7 +41950,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -41975,17 +41975,17 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029313-51gb</t>
+          <t>vivo:VIV202600029313-61gb</t>
         </is>
       </c>
       <c r="H40" s="3" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="I40" s="3" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="4" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
@@ -42022,7 +42022,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -42047,17 +42047,17 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029308-51gb</t>
+          <t>vivo:VIV202600029308-61gb</t>
         </is>
       </c>
       <c r="H41" s="6" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="I41" s="6" t="inlineStr"/>
       <c r="J41" s="5" t="inlineStr"/>
       <c r="K41" s="5" t="inlineStr"/>
       <c r="L41" s="7" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M41" s="5" t="inlineStr">
         <is>
@@ -42094,7 +42094,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -42119,17 +42119,17 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029301-51gb</t>
+          <t>vivo:VIV202600029301-61gb</t>
         </is>
       </c>
       <c r="H42" s="3" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="I42" s="3" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr"/>
       <c r="L42" s="4" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
@@ -42166,7 +42166,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -42191,17 +42191,17 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029274-51gb</t>
+          <t>vivo:VIV202600029274-61gb</t>
         </is>
       </c>
       <c r="H43" s="6" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="I43" s="6" t="inlineStr"/>
       <c r="J43" s="5" t="inlineStr"/>
       <c r="K43" s="5" t="inlineStr"/>
       <c r="L43" s="7" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M43" s="5" t="inlineStr">
         <is>
@@ -42238,7 +42238,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -42263,7 +42263,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600025883-30gb</t>
+          <t>vivo:VIV202600032594-30gb</t>
         </is>
       </c>
       <c r="H44" s="3" t="n">
@@ -42318,7 +42318,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -42343,7 +42343,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600025885-40gb</t>
+          <t>vivo:VIV202600032596-40gb</t>
         </is>
       </c>
       <c r="H45" s="6" t="n">
@@ -42398,7 +42398,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -42423,7 +42423,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600025888-20gb</t>
+          <t>vivo:VIV202600032599-20gb</t>
         </is>
       </c>
       <c r="H46" s="3" t="n">
@@ -42470,7 +42470,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -42542,7 +42542,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -42618,7 +42618,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -42694,7 +42694,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -42770,7 +42770,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -42846,7 +42846,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -42922,7 +42922,7 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
@@ -42994,7 +42994,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -43064,7 +43064,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
@@ -43134,7 +43134,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -43204,7 +43204,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
@@ -43296,7 +43296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -43380,17 +43380,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029273-51gb</t>
+          <t>vivo:VIV202600029274-61gb</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Vivo Controle Educação</t>
+          <t>Vivo Controle Segurança</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="3" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="I2" s="3" t="inlineStr"/>
     </row>
@@ -43407,7 +43407,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>lite</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -43417,17 +43417,17 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029274-51gb</t>
+          <t>vivo:VIV202600032594-30gb</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Vivo Controle Segurança</t>
+          <t>Easy Lite</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr"/>
       <c r="H3" s="6" t="n">
-        <v>85</v>
+        <v>45</v>
       </c>
       <c r="I3" s="6" t="inlineStr"/>
     </row>
@@ -43444,7 +43444,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>lite</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -43454,17 +43454,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029300-51gb</t>
+          <t>vivo:VIV202600032596-40gb</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Vivo Controle</t>
+          <t>Easy Lite</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="3" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="I4" s="3" t="inlineStr"/>
     </row>
@@ -43481,7 +43481,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>lite</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -43491,24 +43491,24 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029301-51gb</t>
+          <t>vivo:VIV202600032599-20gb</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Vivo Controle Saúde</t>
+          <t>Easy Lite</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr"/>
       <c r="H5" s="6" t="n">
-        <v>85</v>
+        <v>35</v>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>removed</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -43518,7 +43518,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>lite</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -43528,24 +43528,24 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029307-51gb</t>
+          <t>vivo:VIV202600025883-30gb</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Vivo Controle Entretenimento</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="n">
-        <v>105</v>
-      </c>
+          <t>Easy Lite</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>removed</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -43555,7 +43555,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>lite</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -43565,24 +43565,24 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029308-51gb</t>
+          <t>vivo:VIV202600025885-40gb</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Vivo Controle Netflix</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="n">
-        <v>90</v>
-      </c>
+          <t>Easy Lite</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>removed</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -43592,7 +43592,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>lite</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -43602,323 +43602,19 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029313-51gb</t>
+          <t>vivo:VIV202600025888-20gb</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Vivo Controle Música</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="3" t="n">
-        <v>90</v>
-      </c>
+          <t>Easy Lite</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>removed</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>vivo</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>control</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>vivo:VIV202600029273-61gb</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Vivo Controle Educação</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>90</v>
-      </c>
-      <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>removed</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>vivo</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>control</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>vivo:VIV202600029300-61gb</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Vivo Controle</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>80</v>
-      </c>
-      <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>removed</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>vivo</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>control</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>vivo:VIV202600029301-61gb</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Vivo Controle Saúde</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>90</v>
-      </c>
-      <c r="H11" s="6" t="inlineStr"/>
-      <c r="I11" s="6" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>removed</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>vivo</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>control</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>vivo:VIV202600029307-61gb</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Vivo Controle Entretenimento</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="n">
-        <v>110</v>
-      </c>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>removed</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>vivo</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>control</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>vivo:VIV202600029308-61gb</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Vivo Controle Netflix</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="n">
-        <v>95</v>
-      </c>
-      <c r="H13" s="6" t="inlineStr"/>
-      <c r="I13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>removed</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>vivo</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>control</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>vivo:VIV202600029313-61gb</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Vivo Controle Música</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="n">
-        <v>95</v>
-      </c>
-      <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>price_change</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>vivo</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>lite</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>vivo:VIV202600025883-30gb</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Easy Lite</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="H15" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="I15" s="6" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>price_change</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>vivo</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>lite</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>vivo:VIV202600025885-40gb</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Easy Lite</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H16" s="3" t="n">
-        <v>55</v>
-      </c>
-      <c r="I16" s="3" t="n">
-        <v>15</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -43957,7 +43653,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01T20:29:30</t>
+          <t>2026-07-01T22:16:09</t>
         </is>
       </c>
     </row>
@@ -44036,7 +43732,7 @@
       </c>
       <c r="D9" s="10">
         <f>IFERROR(AVERAGEIFS(latest!$H$2:$H$2000,latest!$C$2:$C$2000,$A$9),"-")</f>
-        <v>97.09</v>
+        <v>98.68</v>
       </c>
       <c r="E9" s="10">
         <f>IFERROR(_xlfn.MAXIFS(latest!$H$2:$H$2000,latest!$C$2:$C$2000,$A$9),"-")</f>
@@ -45270,7 +44966,7 @@
         <v>2</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>69.90000000000001</v>
@@ -45280,7 +44976,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Vivo Controle (51GB)</t>
+          <t>Vivo Controle (61GB)</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -45299,7 +44995,7 @@
         <v>3</v>
       </c>
       <c r="B17" s="3" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>99.90000000000001</v>
@@ -45309,7 +45005,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Vivo Controle Educação (51GB)</t>
+          <t>Vivo Controle Educação (61GB)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -45328,7 +45024,7 @@
         <v>4</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="6" t="n">
@@ -45336,7 +45032,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Vivo Controle Saúde (51GB)</t>
+          <t>Vivo Controle Saúde (61GB)</t>
         </is>
       </c>
       <c r="F18" s="15" t="n"/>
@@ -45351,14 +45047,14 @@
         <v>5</v>
       </c>
       <c r="B19" s="3" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>84.98999999999999</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Vivo Controle Segurança (51GB)</t>
+          <t>Vivo Controle Segurança (61GB)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -45372,13 +45068,13 @@
         <v>6</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Vivo Controle Música (51GB)</t>
+          <t>Vivo Controle Música (61GB)</t>
         </is>
       </c>
       <c r="F20" s="15" t="n"/>
@@ -45389,11 +45085,11 @@
         <v>7</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Vivo Controle Netflix (51GB)</t>
+          <t>Vivo Controle Netflix (61GB)</t>
         </is>
       </c>
     </row>
@@ -45402,13 +45098,13 @@
         <v>8</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Vivo Controle Entretenimento (51GB)</t>
+          <t>Vivo Controle Entretenimento (61GB)</t>
         </is>
       </c>
       <c r="F22" s="15" t="n"/>
@@ -46125,12 +45821,12 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C12" s="6" t="n"/>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>51 GB (20 GB de franquia 31 GB de bônus)</t>
+          <t>61 GB (20 GB de franquia 31 GB de bônus)</t>
         </is>
       </c>
       <c r="E12" s="5" t="n"/>
@@ -46149,12 +45845,12 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>51 GB (20 GB de franquia 31 GB de bônus)</t>
+          <t>61 GB (20 GB de franquia 31 GB de bônus)</t>
         </is>
       </c>
       <c r="E13" s="2" t="n"/>
@@ -46173,12 +45869,12 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C14" s="6" t="n"/>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>51 GB (20 GB de franquia 31 GB de bônus)</t>
+          <t>61 GB (20 GB de franquia 31 GB de bônus)</t>
         </is>
       </c>
       <c r="E14" s="5" t="n"/>
@@ -46197,12 +45893,12 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>51 GB (20 GB de franquia 31 GB de bônus)</t>
+          <t>61 GB (20 GB de franquia 31 GB de bônus)</t>
         </is>
       </c>
       <c r="E15" s="2" t="n"/>
@@ -46221,12 +45917,12 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C16" s="6" t="n"/>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>51 GB (20 GB de franquia 31 GB de bônus)</t>
+          <t>61 GB (20 GB de franquia 31 GB de bônus)</t>
         </is>
       </c>
       <c r="E16" s="5" t="n"/>
@@ -46245,12 +45941,12 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>51 GB (20 GB de franquia 31 GB de bônus)</t>
+          <t>61 GB (20 GB de franquia 31 GB de bônus)</t>
         </is>
       </c>
       <c r="E17" s="2" t="n"/>
@@ -46269,12 +45965,12 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C18" s="6" t="n"/>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>51 GB (20 GB de franquia 31 GB de bônus)</t>
+          <t>61 GB (20 GB de franquia 31 GB de bônus)</t>
         </is>
       </c>
       <c r="E18" s="5" t="n"/>

</xml_diff>

<commit_message>
chore(data): daily snapshot 2026-07-02
</commit_message>
<xml_diff>
--- a/projects/mobile-price-tracker/data/mobile_plans.xlsx
+++ b/projects/mobile-price-tracker/data/mobile_plans.xlsx
@@ -38770,7 +38770,7 @@
       </c>
       <c r="B531" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C531" s="5" t="inlineStr">
@@ -38848,7 +38848,7 @@
       </c>
       <c r="B532" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C532" s="2" t="inlineStr">
@@ -38920,7 +38920,7 @@
       </c>
       <c r="B533" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C533" s="5" t="inlineStr">
@@ -38992,7 +38992,7 @@
       </c>
       <c r="B534" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C534" s="2" t="inlineStr">
@@ -39064,7 +39064,7 @@
       </c>
       <c r="B535" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C535" s="5" t="inlineStr">
@@ -39136,7 +39136,7 @@
       </c>
       <c r="B536" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C536" s="2" t="inlineStr">
@@ -39208,7 +39208,7 @@
       </c>
       <c r="B537" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C537" s="5" t="inlineStr">
@@ -39280,7 +39280,7 @@
       </c>
       <c r="B538" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C538" s="2" t="inlineStr">
@@ -39352,7 +39352,7 @@
       </c>
       <c r="B539" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C539" s="5" t="inlineStr">
@@ -39424,7 +39424,7 @@
       </c>
       <c r="B540" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C540" s="2" t="inlineStr">
@@ -39496,7 +39496,7 @@
       </c>
       <c r="B541" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C541" s="5" t="inlineStr">
@@ -39568,7 +39568,7 @@
       </c>
       <c r="B542" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C542" s="2" t="inlineStr">
@@ -39640,7 +39640,7 @@
       </c>
       <c r="B543" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C543" s="5" t="inlineStr">
@@ -39710,7 +39710,7 @@
       </c>
       <c r="B544" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C544" s="2" t="inlineStr">
@@ -39780,7 +39780,7 @@
       </c>
       <c r="B545" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C545" s="5" t="inlineStr">
@@ -39850,7 +39850,7 @@
       </c>
       <c r="B546" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C546" s="2" t="inlineStr">
@@ -39920,7 +39920,7 @@
       </c>
       <c r="B547" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C547" s="5" t="inlineStr">
@@ -39990,7 +39990,7 @@
       </c>
       <c r="B548" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C548" s="2" t="inlineStr">
@@ -40060,7 +40060,7 @@
       </c>
       <c r="B549" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C549" s="5" t="inlineStr">
@@ -40130,7 +40130,7 @@
       </c>
       <c r="B550" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C550" s="2" t="inlineStr">
@@ -40194,7 +40194,7 @@
       </c>
       <c r="B551" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C551" s="5" t="inlineStr">
@@ -40258,7 +40258,7 @@
       </c>
       <c r="B552" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C552" s="2" t="inlineStr">
@@ -40322,7 +40322,7 @@
       </c>
       <c r="B553" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C553" s="5" t="inlineStr">
@@ -40386,7 +40386,7 @@
       </c>
       <c r="B554" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C554" s="2" t="inlineStr">
@@ -40448,7 +40448,7 @@
       </c>
       <c r="B555" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C555" s="5" t="inlineStr">
@@ -40516,7 +40516,7 @@
       </c>
       <c r="B556" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C556" s="2" t="inlineStr">
@@ -40584,7 +40584,7 @@
       </c>
       <c r="B557" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C557" s="5" t="inlineStr">
@@ -40652,7 +40652,7 @@
       </c>
       <c r="B558" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C558" s="2" t="inlineStr">
@@ -40720,7 +40720,7 @@
       </c>
       <c r="B559" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C559" s="5" t="inlineStr">
@@ -40788,7 +40788,7 @@
       </c>
       <c r="B560" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C560" s="2" t="inlineStr">
@@ -40856,7 +40856,7 @@
       </c>
       <c r="B561" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C561" s="5" t="inlineStr">
@@ -40924,7 +40924,7 @@
       </c>
       <c r="B562" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C562" s="2" t="inlineStr">
@@ -40990,7 +40990,7 @@
       </c>
       <c r="B563" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C563" s="5" t="inlineStr">
@@ -41056,7 +41056,7 @@
       </c>
       <c r="B564" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C564" s="2" t="inlineStr">
@@ -41122,7 +41122,7 @@
       </c>
       <c r="B565" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C565" s="5" t="inlineStr">
@@ -41194,7 +41194,7 @@
       </c>
       <c r="B566" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C566" s="2" t="inlineStr">
@@ -41219,17 +41219,17 @@
       </c>
       <c r="G566" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029300-61gb</t>
+          <t>vivo:VIV202600029300-51gb</t>
         </is>
       </c>
       <c r="H566" s="3" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="I566" s="3" t="inlineStr"/>
       <c r="J566" s="2" t="inlineStr"/>
       <c r="K566" s="2" t="inlineStr"/>
       <c r="L566" s="4" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M566" s="2" t="inlineStr">
         <is>
@@ -41266,7 +41266,7 @@
       </c>
       <c r="B567" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C567" s="5" t="inlineStr">
@@ -41291,17 +41291,17 @@
       </c>
       <c r="G567" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029273-61gb</t>
+          <t>vivo:VIV202600029273-51gb</t>
         </is>
       </c>
       <c r="H567" s="6" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="I567" s="6" t="inlineStr"/>
       <c r="J567" s="5" t="inlineStr"/>
       <c r="K567" s="5" t="inlineStr"/>
       <c r="L567" s="7" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M567" s="5" t="inlineStr">
         <is>
@@ -41338,7 +41338,7 @@
       </c>
       <c r="B568" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C568" s="2" t="inlineStr">
@@ -41363,17 +41363,17 @@
       </c>
       <c r="G568" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029307-61gb</t>
+          <t>vivo:VIV202600029307-51gb</t>
         </is>
       </c>
       <c r="H568" s="3" t="n">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="I568" s="3" t="inlineStr"/>
       <c r="J568" s="2" t="inlineStr"/>
       <c r="K568" s="2" t="inlineStr"/>
       <c r="L568" s="4" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M568" s="2" t="inlineStr">
         <is>
@@ -41410,7 +41410,7 @@
       </c>
       <c r="B569" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C569" s="5" t="inlineStr">
@@ -41435,17 +41435,17 @@
       </c>
       <c r="G569" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029313-61gb</t>
+          <t>vivo:VIV202600029313-51gb</t>
         </is>
       </c>
       <c r="H569" s="6" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="I569" s="6" t="inlineStr"/>
       <c r="J569" s="5" t="inlineStr"/>
       <c r="K569" s="5" t="inlineStr"/>
       <c r="L569" s="7" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M569" s="5" t="inlineStr">
         <is>
@@ -41482,7 +41482,7 @@
       </c>
       <c r="B570" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C570" s="2" t="inlineStr">
@@ -41507,17 +41507,17 @@
       </c>
       <c r="G570" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029308-61gb</t>
+          <t>vivo:VIV202600029308-51gb</t>
         </is>
       </c>
       <c r="H570" s="3" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="I570" s="3" t="inlineStr"/>
       <c r="J570" s="2" t="inlineStr"/>
       <c r="K570" s="2" t="inlineStr"/>
       <c r="L570" s="4" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M570" s="2" t="inlineStr">
         <is>
@@ -41554,7 +41554,7 @@
       </c>
       <c r="B571" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C571" s="5" t="inlineStr">
@@ -41579,17 +41579,17 @@
       </c>
       <c r="G571" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029301-61gb</t>
+          <t>vivo:VIV202600029301-51gb</t>
         </is>
       </c>
       <c r="H571" s="6" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="I571" s="6" t="inlineStr"/>
       <c r="J571" s="5" t="inlineStr"/>
       <c r="K571" s="5" t="inlineStr"/>
       <c r="L571" s="7" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M571" s="5" t="inlineStr">
         <is>
@@ -41626,7 +41626,7 @@
       </c>
       <c r="B572" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C572" s="2" t="inlineStr">
@@ -41651,17 +41651,17 @@
       </c>
       <c r="G572" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029274-61gb</t>
+          <t>vivo:VIV202600029274-51gb</t>
         </is>
       </c>
       <c r="H572" s="3" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="I572" s="3" t="inlineStr"/>
       <c r="J572" s="2" t="inlineStr"/>
       <c r="K572" s="2" t="inlineStr"/>
       <c r="L572" s="4" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M572" s="2" t="inlineStr">
         <is>
@@ -41698,7 +41698,7 @@
       </c>
       <c r="B573" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C573" s="5" t="inlineStr">
@@ -41778,7 +41778,7 @@
       </c>
       <c r="B574" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C574" s="2" t="inlineStr">
@@ -41858,7 +41858,7 @@
       </c>
       <c r="B575" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C575" s="5" t="inlineStr">
@@ -41930,7 +41930,7 @@
       </c>
       <c r="B576" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C576" s="2" t="inlineStr">
@@ -42002,7 +42002,7 @@
       </c>
       <c r="B577" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C577" s="5" t="inlineStr">
@@ -42078,7 +42078,7 @@
       </c>
       <c r="B578" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C578" s="2" t="inlineStr">
@@ -42154,7 +42154,7 @@
       </c>
       <c r="B579" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C579" s="5" t="inlineStr">
@@ -42230,7 +42230,7 @@
       </c>
       <c r="B580" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C580" s="2" t="inlineStr">
@@ -42306,7 +42306,7 @@
       </c>
       <c r="B581" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C581" s="5" t="inlineStr">
@@ -42382,7 +42382,7 @@
       </c>
       <c r="B582" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C582" s="2" t="inlineStr">
@@ -42454,7 +42454,7 @@
       </c>
       <c r="B583" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C583" s="5" t="inlineStr">
@@ -42524,7 +42524,7 @@
       </c>
       <c r="B584" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C584" s="2" t="inlineStr">
@@ -42594,7 +42594,7 @@
       </c>
       <c r="B585" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C585" s="5" t="inlineStr">
@@ -42664,7 +42664,7 @@
       </c>
       <c r="B586" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C586" s="2" t="inlineStr">
@@ -43327,7 +43327,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -43405,7 +43405,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -43477,7 +43477,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -43549,7 +43549,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -43621,7 +43621,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -43693,7 +43693,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -43765,7 +43765,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -43837,7 +43837,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -43909,7 +43909,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -43981,7 +43981,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -44053,7 +44053,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -44125,7 +44125,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -44197,7 +44197,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -44267,7 +44267,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -44337,7 +44337,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -44477,7 +44477,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -44547,7 +44547,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -44617,7 +44617,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -44687,7 +44687,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -44751,7 +44751,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -44815,7 +44815,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -44879,7 +44879,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -44943,7 +44943,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -45005,7 +45005,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -45073,7 +45073,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -45141,7 +45141,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -45209,7 +45209,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -45277,7 +45277,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -45345,7 +45345,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -45413,7 +45413,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -45481,7 +45481,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -45547,7 +45547,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -45613,7 +45613,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -45679,7 +45679,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -45751,7 +45751,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -45776,17 +45776,17 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029300-61gb</t>
+          <t>vivo:VIV202600029300-51gb</t>
         </is>
       </c>
       <c r="H37" s="6" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="I37" s="6" t="inlineStr"/>
       <c r="J37" s="5" t="inlineStr"/>
       <c r="K37" s="5" t="inlineStr"/>
       <c r="L37" s="7" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M37" s="5" t="inlineStr">
         <is>
@@ -45823,7 +45823,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -45848,17 +45848,17 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029273-61gb</t>
+          <t>vivo:VIV202600029273-51gb</t>
         </is>
       </c>
       <c r="H38" s="3" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="I38" s="3" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="4" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
@@ -45895,7 +45895,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -45920,17 +45920,17 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029307-61gb</t>
+          <t>vivo:VIV202600029307-51gb</t>
         </is>
       </c>
       <c r="H39" s="6" t="n">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="I39" s="6" t="inlineStr"/>
       <c r="J39" s="5" t="inlineStr"/>
       <c r="K39" s="5" t="inlineStr"/>
       <c r="L39" s="7" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M39" s="5" t="inlineStr">
         <is>
@@ -45967,7 +45967,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -45992,17 +45992,17 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029313-61gb</t>
+          <t>vivo:VIV202600029313-51gb</t>
         </is>
       </c>
       <c r="H40" s="3" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="I40" s="3" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="4" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
@@ -46039,7 +46039,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -46064,17 +46064,17 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029308-61gb</t>
+          <t>vivo:VIV202600029308-51gb</t>
         </is>
       </c>
       <c r="H41" s="6" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="I41" s="6" t="inlineStr"/>
       <c r="J41" s="5" t="inlineStr"/>
       <c r="K41" s="5" t="inlineStr"/>
       <c r="L41" s="7" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M41" s="5" t="inlineStr">
         <is>
@@ -46111,7 +46111,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -46136,17 +46136,17 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029301-61gb</t>
+          <t>vivo:VIV202600029301-51gb</t>
         </is>
       </c>
       <c r="H42" s="3" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="I42" s="3" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr"/>
       <c r="L42" s="4" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
@@ -46183,7 +46183,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -46208,17 +46208,17 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>vivo:VIV202600029274-61gb</t>
+          <t>vivo:VIV202600029274-51gb</t>
         </is>
       </c>
       <c r="H43" s="6" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="I43" s="6" t="inlineStr"/>
       <c r="J43" s="5" t="inlineStr"/>
       <c r="K43" s="5" t="inlineStr"/>
       <c r="L43" s="7" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M43" s="5" t="inlineStr">
         <is>
@@ -46255,7 +46255,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -46335,7 +46335,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -46415,7 +46415,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -46487,7 +46487,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -46559,7 +46559,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -46635,7 +46635,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -46711,7 +46711,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -46787,7 +46787,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -46863,7 +46863,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -46939,7 +46939,7 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
@@ -47011,7 +47011,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -47081,7 +47081,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
@@ -47151,7 +47151,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -47221,7 +47221,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
@@ -47313,7 +47313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -47373,6 +47373,524 @@
           <t>delta_brl</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029273-51gb</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle Educação</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr"/>
+      <c r="H2" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="I2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029274-51gb</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Controle Segurança</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr"/>
+      <c r="H3" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="I3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029300-51gb</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="n">
+        <v>75</v>
+      </c>
+      <c r="I4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029301-51gb</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Controle Saúde</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="I5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029307-51gb</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle Entretenimento</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="n">
+        <v>105</v>
+      </c>
+      <c r="I6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029308-51gb</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Controle Netflix</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="I7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029313-51gb</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle Música</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="I8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029273-61gb</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Controle Educação</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029274-61gb</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle Segurança</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029300-61gb</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Controle</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="H11" s="6" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029301-61gb</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle Saúde</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="H12" s="3" t="inlineStr"/>
+      <c r="I12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029307-61gb</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Controle Entretenimento</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>110</v>
+      </c>
+      <c r="H13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029308-61gb</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle Netflix</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>removed</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>vivo:VIV202600029313-61gb</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Vivo Controle Música</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -47411,7 +47929,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-02T17:51:26</t>
+          <t>2026-07-02T22:04:41</t>
         </is>
       </c>
     </row>
@@ -47490,7 +48008,7 @@
       </c>
       <c r="D9" s="10">
         <f>IFERROR(AVERAGEIFS(latest!$H$2:$H$2000,latest!$C$2:$C$2000,$A$9),"-")</f>
-        <v>98.68</v>
+        <v>97.09</v>
       </c>
       <c r="E9" s="10">
         <f>IFERROR(_xlfn.MAXIFS(latest!$H$2:$H$2000,latest!$C$2:$C$2000,$A$9),"-")</f>
@@ -48784,7 +49302,7 @@
         <v>2</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>69.90000000000001</v>
@@ -48794,7 +49312,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Vivo Controle (61GB)</t>
+          <t>Vivo Controle (51GB)</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -48813,7 +49331,7 @@
         <v>3</v>
       </c>
       <c r="B17" s="3" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>99.90000000000001</v>
@@ -48823,7 +49341,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Vivo Controle Educação (61GB)</t>
+          <t>Vivo Controle Educação (51GB)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -48842,7 +49360,7 @@
         <v>4</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="6" t="n">
@@ -48850,7 +49368,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Vivo Controle Saúde (61GB)</t>
+          <t>Vivo Controle Saúde (51GB)</t>
         </is>
       </c>
       <c r="F18" s="15" t="n"/>
@@ -48865,14 +49383,14 @@
         <v>5</v>
       </c>
       <c r="B19" s="3" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>84.98999999999999</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Vivo Controle Segurança (61GB)</t>
+          <t>Vivo Controle Segurança (51GB)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -48886,13 +49404,13 @@
         <v>6</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Vivo Controle Música (61GB)</t>
+          <t>Vivo Controle Música (51GB)</t>
         </is>
       </c>
       <c r="F20" s="15" t="n"/>
@@ -48903,11 +49421,11 @@
         <v>7</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Vivo Controle Netflix (61GB)</t>
+          <t>Vivo Controle Netflix (51GB)</t>
         </is>
       </c>
     </row>
@@ -48916,13 +49434,13 @@
         <v>8</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Vivo Controle Entretenimento (61GB)</t>
+          <t>Vivo Controle Entretenimento (51GB)</t>
         </is>
       </c>
       <c r="F22" s="15" t="n"/>
@@ -49639,12 +50157,12 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C12" s="6" t="n"/>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>61 GB (20 GB de franquia 31 GB de bônus)</t>
+          <t>51 GB (20 GB de franquia 31 GB de bônus)</t>
         </is>
       </c>
       <c r="E12" s="5" t="n"/>
@@ -49663,12 +50181,12 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>61 GB (20 GB de franquia 31 GB de bônus)</t>
+          <t>51 GB (20 GB de franquia 31 GB de bônus)</t>
         </is>
       </c>
       <c r="E13" s="2" t="n"/>
@@ -49687,12 +50205,12 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C14" s="6" t="n"/>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>61 GB (20 GB de franquia 31 GB de bônus)</t>
+          <t>51 GB (20 GB de franquia 31 GB de bônus)</t>
         </is>
       </c>
       <c r="E14" s="5" t="n"/>
@@ -49711,12 +50229,12 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>61 GB (20 GB de franquia 31 GB de bônus)</t>
+          <t>51 GB (20 GB de franquia 31 GB de bônus)</t>
         </is>
       </c>
       <c r="E15" s="2" t="n"/>
@@ -49735,12 +50253,12 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C16" s="6" t="n"/>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>61 GB (20 GB de franquia 31 GB de bônus)</t>
+          <t>51 GB (20 GB de franquia 31 GB de bônus)</t>
         </is>
       </c>
       <c r="E16" s="5" t="n"/>
@@ -49759,12 +50277,12 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>61 GB (20 GB de franquia 31 GB de bônus)</t>
+          <t>51 GB (20 GB de franquia 31 GB de bônus)</t>
         </is>
       </c>
       <c r="E17" s="2" t="n"/>
@@ -49783,12 +50301,12 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C18" s="6" t="n"/>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>61 GB (20 GB de franquia 31 GB de bônus)</t>
+          <t>51 GB (20 GB de franquia 31 GB de bônus)</t>
         </is>
       </c>
       <c r="E18" s="5" t="n"/>

</xml_diff>

<commit_message>
chore(data): daily snapshot 2026-07-03
</commit_message>
<xml_diff>
--- a/projects/mobile-price-tracker/data/mobile_plans.xlsx
+++ b/projects/mobile-price-tracker/data/mobile_plans.xlsx
@@ -42734,7 +42734,7 @@
       </c>
       <c r="B587" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C587" s="5" t="inlineStr">
@@ -42812,7 +42812,7 @@
       </c>
       <c r="B588" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C588" s="2" t="inlineStr">
@@ -42884,7 +42884,7 @@
       </c>
       <c r="B589" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C589" s="5" t="inlineStr">
@@ -42956,7 +42956,7 @@
       </c>
       <c r="B590" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C590" s="2" t="inlineStr">
@@ -43028,7 +43028,7 @@
       </c>
       <c r="B591" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C591" s="5" t="inlineStr">
@@ -43100,7 +43100,7 @@
       </c>
       <c r="B592" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C592" s="2" t="inlineStr">
@@ -43172,7 +43172,7 @@
       </c>
       <c r="B593" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C593" s="5" t="inlineStr">
@@ -43244,7 +43244,7 @@
       </c>
       <c r="B594" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C594" s="2" t="inlineStr">
@@ -43316,7 +43316,7 @@
       </c>
       <c r="B595" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C595" s="5" t="inlineStr">
@@ -43388,7 +43388,7 @@
       </c>
       <c r="B596" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C596" s="2" t="inlineStr">
@@ -43460,7 +43460,7 @@
       </c>
       <c r="B597" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C597" s="5" t="inlineStr">
@@ -43532,7 +43532,7 @@
       </c>
       <c r="B598" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C598" s="2" t="inlineStr">
@@ -43604,7 +43604,7 @@
       </c>
       <c r="B599" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C599" s="5" t="inlineStr">
@@ -43674,7 +43674,7 @@
       </c>
       <c r="B600" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C600" s="2" t="inlineStr">
@@ -43744,7 +43744,7 @@
       </c>
       <c r="B601" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C601" s="5" t="inlineStr">
@@ -43814,7 +43814,7 @@
       </c>
       <c r="B602" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C602" s="2" t="inlineStr">
@@ -43884,7 +43884,7 @@
       </c>
       <c r="B603" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C603" s="5" t="inlineStr">
@@ -43954,7 +43954,7 @@
       </c>
       <c r="B604" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C604" s="2" t="inlineStr">
@@ -44024,7 +44024,7 @@
       </c>
       <c r="B605" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C605" s="5" t="inlineStr">
@@ -44094,7 +44094,7 @@
       </c>
       <c r="B606" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C606" s="2" t="inlineStr">
@@ -44158,7 +44158,7 @@
       </c>
       <c r="B607" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C607" s="5" t="inlineStr">
@@ -44222,7 +44222,7 @@
       </c>
       <c r="B608" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C608" s="2" t="inlineStr">
@@ -44286,7 +44286,7 @@
       </c>
       <c r="B609" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C609" s="5" t="inlineStr">
@@ -44350,7 +44350,7 @@
       </c>
       <c r="B610" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C610" s="2" t="inlineStr">
@@ -44412,7 +44412,7 @@
       </c>
       <c r="B611" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C611" s="5" t="inlineStr">
@@ -44480,7 +44480,7 @@
       </c>
       <c r="B612" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C612" s="2" t="inlineStr">
@@ -44548,7 +44548,7 @@
       </c>
       <c r="B613" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C613" s="5" t="inlineStr">
@@ -44616,7 +44616,7 @@
       </c>
       <c r="B614" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C614" s="2" t="inlineStr">
@@ -44684,7 +44684,7 @@
       </c>
       <c r="B615" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C615" s="5" t="inlineStr">
@@ -44752,7 +44752,7 @@
       </c>
       <c r="B616" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C616" s="2" t="inlineStr">
@@ -44820,7 +44820,7 @@
       </c>
       <c r="B617" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C617" s="5" t="inlineStr">
@@ -44888,7 +44888,7 @@
       </c>
       <c r="B618" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C618" s="2" t="inlineStr">
@@ -44954,7 +44954,7 @@
       </c>
       <c r="B619" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C619" s="5" t="inlineStr">
@@ -45020,7 +45020,7 @@
       </c>
       <c r="B620" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C620" s="2" t="inlineStr">
@@ -45086,7 +45086,7 @@
       </c>
       <c r="B621" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C621" s="5" t="inlineStr">
@@ -45158,7 +45158,7 @@
       </c>
       <c r="B622" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C622" s="2" t="inlineStr">
@@ -45230,7 +45230,7 @@
       </c>
       <c r="B623" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C623" s="5" t="inlineStr">
@@ -45302,7 +45302,7 @@
       </c>
       <c r="B624" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C624" s="2" t="inlineStr">
@@ -45374,7 +45374,7 @@
       </c>
       <c r="B625" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C625" s="5" t="inlineStr">
@@ -45446,7 +45446,7 @@
       </c>
       <c r="B626" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C626" s="2" t="inlineStr">
@@ -45518,7 +45518,7 @@
       </c>
       <c r="B627" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C627" s="5" t="inlineStr">
@@ -45590,7 +45590,7 @@
       </c>
       <c r="B628" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C628" s="2" t="inlineStr">
@@ -45662,7 +45662,7 @@
       </c>
       <c r="B629" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C629" s="5" t="inlineStr">
@@ -45742,7 +45742,7 @@
       </c>
       <c r="B630" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C630" s="2" t="inlineStr">
@@ -45822,7 +45822,7 @@
       </c>
       <c r="B631" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C631" s="5" t="inlineStr">
@@ -45894,7 +45894,7 @@
       </c>
       <c r="B632" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C632" s="2" t="inlineStr">
@@ -45966,7 +45966,7 @@
       </c>
       <c r="B633" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C633" s="5" t="inlineStr">
@@ -46042,7 +46042,7 @@
       </c>
       <c r="B634" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C634" s="2" t="inlineStr">
@@ -46118,7 +46118,7 @@
       </c>
       <c r="B635" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C635" s="5" t="inlineStr">
@@ -46194,7 +46194,7 @@
       </c>
       <c r="B636" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C636" s="2" t="inlineStr">
@@ -46270,7 +46270,7 @@
       </c>
       <c r="B637" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C637" s="5" t="inlineStr">
@@ -46346,7 +46346,7 @@
       </c>
       <c r="B638" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C638" s="2" t="inlineStr">
@@ -46418,7 +46418,7 @@
       </c>
       <c r="B639" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C639" s="5" t="inlineStr">
@@ -46488,7 +46488,7 @@
       </c>
       <c r="B640" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C640" s="2" t="inlineStr">
@@ -46558,7 +46558,7 @@
       </c>
       <c r="B641" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C641" s="5" t="inlineStr">
@@ -46628,7 +46628,7 @@
       </c>
       <c r="B642" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C642" s="2" t="inlineStr">
@@ -47291,7 +47291,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -47369,7 +47369,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -47441,7 +47441,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -47513,7 +47513,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -47585,7 +47585,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -47657,7 +47657,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -47729,7 +47729,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -47801,7 +47801,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -47873,7 +47873,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -47945,7 +47945,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -48017,7 +48017,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -48089,7 +48089,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -48161,7 +48161,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -48231,7 +48231,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -48301,7 +48301,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -48371,7 +48371,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -48441,7 +48441,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -48511,7 +48511,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -48581,7 +48581,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -48651,7 +48651,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -48715,7 +48715,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -48779,7 +48779,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -48843,7 +48843,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -48907,7 +48907,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -48969,7 +48969,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -49037,7 +49037,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -49105,7 +49105,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -49173,7 +49173,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -49241,7 +49241,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -49309,7 +49309,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -49377,7 +49377,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -49445,7 +49445,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -49511,7 +49511,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -49577,7 +49577,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -49643,7 +49643,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -49715,7 +49715,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -49787,7 +49787,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -49859,7 +49859,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -49931,7 +49931,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -50003,7 +50003,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -50075,7 +50075,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -50147,7 +50147,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -50219,7 +50219,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -50299,7 +50299,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -50379,7 +50379,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -50451,7 +50451,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -50523,7 +50523,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -50599,7 +50599,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -50675,7 +50675,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -50751,7 +50751,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -50827,7 +50827,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -50903,7 +50903,7 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
@@ -50975,7 +50975,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -51045,7 +51045,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
@@ -51115,7 +51115,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -51185,7 +51185,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
@@ -51893,7 +51893,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03T17:00:50</t>
+          <t>2026-07-03T22:03:07</t>
         </is>
       </c>
     </row>

</xml_diff>